<commit_message>
Grab Thailand: 5-market depth cascade, sheet publish, deck KPI refresh
Expand economics to eastern_seaboard + royal_coast with depth/Ko Lanta
corridors; relink upper-Gulf journeys. Cascade now covers 26 routes,
$240M pool, $25M SOM floor, $529M SAM, $2.11B marine TAM.

Publish unit-economics sheet to Drive; bind 17 Bucket-C mesh legs.
Apply refreshed KPIs and TAM ladder to live Slides deck; add economics
value sidecar and market-scope.json.
</commit_message>
<xml_diff>
--- a/finance/_refresh_grab-thailand.xlsx
+++ b/finance/_refresh_grab-thailand.xlsx
@@ -45,8 +45,8 @@
     <definedName name="load_sel">'Assumptions'!$B$39</definedName>
     <definedName name="revleg_sel">'Assumptions'!$B$40</definedName>
     <definedName name="country_opex">'Country opex'!$A$4:$G$4</definedName>
-    <definedName name="som_floor_fleet">'Corridor economics'!$D$26</definedName>
-    <definedName name="som_floor_rev">'Corridor economics'!$E$26</definedName>
+    <definedName name="som_floor_fleet">'Corridor economics'!$D$39</definedName>
+    <definedName name="som_floor_rev">'Corridor economics'!$E$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1919,7 +1919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY29"/>
+  <dimension ref="A1:AY42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2447,7 +2447,7 @@
     <row r="5">
       <c r="A5" s="29" t="inlineStr">
         <is>
-          <t>Bangkok</t>
+          <t>Eastern_Seaboard</t>
         </is>
       </c>
       <c r="B5" s="29" t="inlineStr">
@@ -2457,23 +2457,23 @@
       </c>
       <c r="C5" s="30" t="inlineStr">
         <is>
-          <t>ICONSIAM Pier (Chao Phraya) → ICONSIAM Pier (Chao Phraya)</t>
+          <t>Ban Phe Pier → Koh Samet (Na Dan Pier)</t>
         </is>
       </c>
       <c r="D5" s="31" t="n">
-        <v>5.3</v>
+        <v>3.3</v>
       </c>
       <c r="E5" s="26" t="n">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="F5" s="32" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T5</t>
         </is>
       </c>
       <c r="G5" s="32" t="inlineStr">
         <is>
-          <t>med</t>
+          <t>low-med</t>
         </is>
       </c>
       <c r="H5" s="19" t="n">
@@ -2576,10 +2576,18 @@
         <v/>
       </c>
       <c r="AG5" s="31" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="AH5" s="32" t="n"/>
-      <c r="AI5" s="32" t="n"/>
+        <v>92000</v>
+      </c>
+      <c r="AH5" s="32" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="AI5" s="32" t="inlineStr">
+        <is>
+          <t>low-med</t>
+        </is>
+      </c>
       <c r="AJ5" s="39" t="n">
         <v>0.1</v>
       </c>
@@ -2626,15 +2634,19 @@
       </c>
       <c r="AX5" s="44" t="inlineStr">
         <is>
-          <t>Conservative mid of the live Jun-2026 promo band across 24 listed dinner-round products (899-2,000 THB; cluster at 1,150-1,550): click2gothailand.com top-10 guide (updated 1-Jun-2026); Bangkok Chaophraya Cruise operator site lists 1,550 THB/pax rack. Navier 8-pax product would be drinks/canape-class, not galley-buffet-class, hence mid-band anchor not premium.</t>
-        </is>
-      </c>
-      <c r="AY5" s="44" t="n"/>
+          <t>Proven high-frequency Ban Phe speedboat gateway; premium upgrade of dense leg.</t>
+        </is>
+      </c>
+      <c r="AY5" s="44" t="inlineStr">
+        <is>
+          <t>Proven high-frequency Ban Phe speedboat gateway; premium upgrade of dense leg.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="29" t="inlineStr">
         <is>
-          <t>Koh Samui</t>
+          <t>Bangkok</t>
         </is>
       </c>
       <c r="B6" s="29" t="inlineStr">
@@ -2644,19 +2656,23 @@
       </c>
       <c r="C6" s="30" t="inlineStr">
         <is>
-          <t>Samui Pralarn Pier (Mae Nam) → Koh Phangan (Thong Sala) — pier-exact</t>
+          <t>ICONSIAM Pier (Chao Phraya) → ICONSIAM Pier (Chao Phraya)</t>
         </is>
       </c>
       <c r="D6" s="31" t="n">
-        <v>7.5</v>
+        <v>5.3</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>35</v>
       </c>
-      <c r="F6" s="32" t="n"/>
+      <c r="F6" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
       <c r="G6" s="32" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>med</t>
         </is>
       </c>
       <c r="H6" s="19" t="n">
@@ -2759,18 +2775,10 @@
         <v/>
       </c>
       <c r="AG6" s="31" t="n">
-        <v>450000</v>
-      </c>
-      <c r="AH6" s="32" t="inlineStr">
-        <is>
-          <t>T5</t>
-        </is>
-      </c>
-      <c r="AI6" s="32" t="inlineStr">
-        <is>
-          <t>low-med</t>
-        </is>
-      </c>
+        <v>1200000</v>
+      </c>
+      <c r="AH6" s="32" t="n"/>
+      <c r="AI6" s="32" t="n"/>
       <c r="AJ6" s="39" t="n">
         <v>0.1</v>
       </c>
@@ -2794,11 +2802,7 @@
         <f>IF(AN6="","",AN6*T6)</f>
         <v/>
       </c>
-      <c r="AP6" s="40" t="inlineStr">
-        <is>
-          <t>rn-db5e83248f9d</t>
-        </is>
-      </c>
+      <c r="AP6" s="40" t="n"/>
       <c r="AQ6" s="32" t="inlineStr">
         <is>
           <t>Grounded</t>
@@ -2819,17 +2823,17 @@
         <f>IF(((S6*pax_cap*load_full*ROUND(K6*L6*revleg_full,0))-(((battery/range_nm)*D6*ROUND(K6*L6*revleg_full,0)*VLOOKUP(B6,country_opex,3,FALSE))+V6+W6+X6+Y6+Z6))&lt;=0,"",VLOOKUP(B6,country_opex,7,FALSE)/((S6*pax_cap*load_full*ROUND(K6*L6*revleg_full,0))-(((battery/range_nm)*D6*ROUND(K6*L6*revleg_full,0)*VLOOKUP(B6,country_opex,3,FALSE))+V6+W6+X6+Y6+Z6)))</f>
         <v/>
       </c>
-      <c r="AX6" s="44" t="n"/>
-      <c r="AY6" s="44" t="inlineStr">
-        <is>
-          <t>SUBSET of rn-db5e83248f9d (do not sum). Lomprayah operates the Pralarn (Mae Nam) terminal with ~4-6 daily fast-cat departures/direction to Thong Sala (lomprayah.com 2026 timetable; ferryadvice.com: Pralarn-&gt;Thong Sala 20 min, THB 300); Lomprayah is the highest-frequency operator on the crossing.</t>
-        </is>
-      </c>
+      <c r="AX6" s="44" t="inlineStr">
+        <is>
+          <t>Conservative mid of the live Jun-2026 promo band across 24 listed dinner-round products (899-2,000 THB; cluster at 1,150-1,550): click2gothailand.com top-10 guide (updated 1-Jun-2026); Bangkok Chaophraya Cruise operator site lists 1,550 THB/pax rack. Navier 8-pax product would be drinks/canape-class, not galley-buffet-class, hence mid-band anchor not premium.</t>
+        </is>
+      </c>
+      <c r="AY6" s="44" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="29" t="inlineStr">
         <is>
-          <t>Phuket</t>
+          <t>Koh Samui</t>
         </is>
       </c>
       <c r="B7" s="29" t="inlineStr">
@@ -2839,23 +2843,19 @@
       </c>
       <c r="C7" s="30" t="inlineStr">
         <is>
-          <t>Chalong Pier (Ao Chalong) → Chalong Pier (Ao Chalong)</t>
+          <t>Samui Pralarn Pier (Mae Nam) → Koh Phangan (Thong Sala) — pier-exact</t>
         </is>
       </c>
       <c r="D7" s="31" t="n">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="E7" s="26" t="n">
         <v>35</v>
       </c>
-      <c r="F7" s="32" t="inlineStr">
+      <c r="F7" s="32" t="n"/>
+      <c r="G7" s="32" t="inlineStr">
         <is>
           <t>T1</t>
-        </is>
-      </c>
-      <c r="G7" s="32" t="inlineStr">
-        <is>
-          <t>med</t>
         </is>
       </c>
       <c r="H7" s="19" t="n">
@@ -2958,10 +2958,18 @@
         <v/>
       </c>
       <c r="AG7" s="31" t="n">
-        <v>400000</v>
-      </c>
-      <c r="AH7" s="32" t="n"/>
-      <c r="AI7" s="32" t="n"/>
+        <v>450000</v>
+      </c>
+      <c r="AH7" s="32" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
+      <c r="AI7" s="32" t="inlineStr">
+        <is>
+          <t>low-med</t>
+        </is>
+      </c>
       <c r="AJ7" s="39" t="n">
         <v>0.1</v>
       </c>
@@ -2985,7 +2993,11 @@
         <f>IF(AN7="","",AN7*T7)</f>
         <v/>
       </c>
-      <c r="AP7" s="40" t="n"/>
+      <c r="AP7" s="40" t="inlineStr">
+        <is>
+          <t>rn-db5e83248f9d</t>
+        </is>
+      </c>
       <c r="AQ7" s="32" t="inlineStr">
         <is>
           <t>Grounded</t>
@@ -3006,17 +3018,17 @@
         <f>IF(((S7*pax_cap*load_full*ROUND(K7*L7*revleg_full,0))-(((battery/range_nm)*D7*ROUND(K7*L7*revleg_full,0)*VLOOKUP(B7,country_opex,3,FALSE))+V7+W7+X7+Y7+Z7))&lt;=0,"",VLOOKUP(B7,country_opex,7,FALSE)/((S7*pax_cap*load_full*ROUND(K7*L7*revleg_full,0))-(((battery/range_nm)*D7*ROUND(K7*L7*revleg_full,0)*VLOOKUP(B7,country_opex,3,FALSE))+V7+W7+X7+Y7+Z7)))</f>
         <v/>
       </c>
-      <c r="AX7" s="44" t="inlineStr">
-        <is>
-          <t>Modal product = shared speedboat Coral Island half/one-day trip ex-Chalong: Love Sea Tour Racha+Coral speedboat 1,200 THB adult (promo 1,050) (loveseatour.com/racha-coral-speed-boat/); JC Tour Coral+snorkel 1,200 THB (jctour-thai.com/coral); Andamarine one-day Racha Yai+Coral 1,250 THB/pax incl. buffet lunch (operator IG, 2026). Premium top of ladder: HYPE join-in day cruise 3,900 THB adult incl. transfer (operator rate sheet via boatingo.com/boats/hype-catamaran/). Anchor = modal speedboat product ~1,250 THB = ~USD 35, NOT the premium cat.</t>
-        </is>
-      </c>
-      <c r="AY7" s="44" t="n"/>
+      <c r="AX7" s="44" t="n"/>
+      <c r="AY7" s="44" t="inlineStr">
+        <is>
+          <t>SUBSET of rn-db5e83248f9d (do not sum). Lomprayah operates the Pralarn (Mae Nam) terminal with ~4-6 daily fast-cat departures/direction to Thong Sala (lomprayah.com 2026 timetable; ferryadvice.com: Pralarn-&gt;Thong Sala 20 min, THB 300); Lomprayah is the highest-frequency operator on the crossing.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="29" t="inlineStr">
         <is>
-          <t>Koh Samui</t>
+          <t>Phuket</t>
         </is>
       </c>
       <c r="B8" s="29" t="inlineStr">
@@ -3026,19 +3038,23 @@
       </c>
       <c r="C8" s="30" t="inlineStr">
         <is>
-          <t>Koh Samui (Bangrak) → Koh Phangan (Thong Sala)</t>
+          <t>Ao Po Grand Marina → Anantara Layan Phuket Beach Jetty</t>
         </is>
       </c>
       <c r="D8" s="31" t="n">
-        <v>10.2</v>
+        <v>9.6</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>10</v>
-      </c>
-      <c r="F8" s="32" t="n"/>
+        <v>100</v>
+      </c>
+      <c r="F8" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
       <c r="G8" s="32" t="inlineStr">
         <is>
-          <t>derived_pending_validation</t>
+          <t>med</t>
         </is>
       </c>
       <c r="H8" s="19" t="n">
@@ -3141,16 +3157,20 @@
         <v/>
       </c>
       <c r="AG8" s="31" t="n">
-        <v>19404</v>
-      </c>
-      <c r="AH8" s="32" t="n"/>
+        <v>8500</v>
+      </c>
+      <c r="AH8" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
       <c r="AI8" s="32" t="inlineStr">
         <is>
-          <t>derived_pending_validation</t>
+          <t>med</t>
         </is>
       </c>
       <c r="AJ8" s="39" t="n">
-        <v>0.1</v>
+        <v>0.9</v>
       </c>
       <c r="AK8" s="34">
         <f>IF(AG8="","",AG8*AJ8)</f>
@@ -3195,12 +3215,12 @@
       </c>
       <c r="AX8" s="44" t="inlineStr">
         <is>
-          <t>Koh Samui (Bangrak/Maenam) -&gt; Koh Phangan (Thong Sala)</t>
+          <t>Minor Hotels captive gateway — Anantara Layan marina pickup.</t>
         </is>
       </c>
       <c r="AY8" s="44" t="inlineStr">
         <is>
-          <t>Koh Samui (Bangrak/Maenam) -&gt; Koh Phangan (Thong Sala)</t>
+          <t>minor-hotels-phuket-flagship-economics-DRAFT.json — Layan gateway pool</t>
         </is>
       </c>
     </row>
@@ -3217,18 +3237,18 @@
       </c>
       <c r="C9" s="30" t="inlineStr">
         <is>
-          <t>Ao Po Pier (Ao Po / Ao Por, NE Phuket) → Khao Phing Kan (James Bond Island), Phang Nga Bay</t>
+          <t>Chalong Pier (Ao Chalong) → Chalong Pier (Ao Chalong)</t>
         </is>
       </c>
       <c r="D9" s="31" t="n">
-        <v>13.5</v>
+        <v>10</v>
       </c>
       <c r="E9" s="26" t="n">
-        <v>90</v>
+        <v>35</v>
       </c>
       <c r="F9" s="32" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="G9" s="32" t="inlineStr">
@@ -3336,7 +3356,7 @@
         <v/>
       </c>
       <c r="AG9" s="31" t="n">
-        <v>20000</v>
+        <v>400000</v>
       </c>
       <c r="AH9" s="32" t="n"/>
       <c r="AI9" s="32" t="n"/>
@@ -3386,7 +3406,7 @@
       </c>
       <c r="AX9" s="44" t="inlineStr">
         <is>
-          <t>John Gray's Hong by Starlight 3,350 THB/pax agent rate (phukettoursdirect.com/hong-by-starlight.html) / USD 108.89 retail (Agoda activities listing); Phuket Sail Tours sunset/day band 2,200-2,800 THB (phuketexpatguide.com operator comparison, 2026); Simba Sea Trips premium small-group products (TripAdvisor-listed, 18-adult cap, award-positioned above mass market). Anchor = conservative mid of the 2,500-3,900 THB premium band ~ USD 90.</t>
+          <t>Modal product = shared speedboat Coral Island half/one-day trip ex-Chalong: Love Sea Tour Racha+Coral speedboat 1,200 THB adult (promo 1,050) (loveseatour.com/racha-coral-speed-boat/); JC Tour Coral+snorkel 1,200 THB (jctour-thai.com/coral); Andamarine one-day Racha Yai+Coral 1,250 THB/pax incl. buffet lunch (operator IG, 2026). Premium top of ladder: HYPE join-in day cruise 3,900 THB adult incl. transfer (operator rate sheet via boatingo.com/boats/hype-catamaran/). Anchor = modal speedboat product ~1,250 THB = ~USD 35, NOT the premium cat.</t>
         </is>
       </c>
       <c r="AY9" s="44" t="n"/>
@@ -3404,19 +3424,19 @@
       </c>
       <c r="C10" s="30" t="inlineStr">
         <is>
-          <t>Koh Samui (Lipa Noi) → Donsak (Raja Ferry pier)</t>
+          <t>Koh Samui (Bangrak) → Koh Phangan (Thong Sala)</t>
         </is>
       </c>
       <c r="D10" s="31" t="n">
-        <v>14.3</v>
+        <v>10.2</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>15.2</v>
+        <v>10</v>
       </c>
       <c r="F10" s="32" t="n"/>
       <c r="G10" s="32" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>derived_pending_validation</t>
         </is>
       </c>
       <c r="H10" s="19" t="n">
@@ -3431,7 +3451,7 @@
         <v/>
       </c>
       <c r="K10" s="34">
-        <f>MIN(24,FLOOR(60*service_hr/J10,1))</f>
+        <f>MIN(15,FLOOR(60*service_hr/J10,1))</f>
         <v/>
       </c>
       <c r="L10" s="34">
@@ -3519,16 +3539,12 @@
         <v/>
       </c>
       <c r="AG10" s="31" t="n">
-        <v>666667</v>
-      </c>
-      <c r="AH10" s="32" t="inlineStr">
-        <is>
-          <t>T2</t>
-        </is>
-      </c>
+        <v>19404</v>
+      </c>
+      <c r="AH10" s="32" t="n"/>
       <c r="AI10" s="32" t="inlineStr">
         <is>
-          <t>med-low</t>
+          <t>derived_pending_validation</t>
         </is>
       </c>
       <c r="AJ10" s="39" t="n">
@@ -3575,17 +3591,21 @@
         <f>IF(((S10*pax_cap*load_full*ROUND(K10*L10*revleg_full,0))-(((battery/range_nm)*D10*ROUND(K10*L10*revleg_full,0)*VLOOKUP(B10,country_opex,3,FALSE))+V10+W10+X10+Y10+Z10))&lt;=0,"",VLOOKUP(B10,country_opex,7,FALSE)/((S10*pax_cap*load_full*ROUND(K10*L10*revleg_full,0))-(((battery/range_nm)*D10*ROUND(K10*L10*revleg_full,0)*VLOOKUP(B10,country_opex,3,FALSE))+V10+W10+X10+Y10+Z10)))</f>
         <v/>
       </c>
-      <c r="AX10" s="44" t="n"/>
+      <c r="AX10" s="44" t="inlineStr">
+        <is>
+          <t>Koh Samui (Bangrak/Maenam) -&gt; Koh Phangan (Thong Sala)</t>
+        </is>
+      </c>
       <c r="AY10" s="44" t="inlineStr">
         <is>
-          <t>SUBSET of rn-347c44e1d360 (do not sum). Raja Ferry Port (SET-listed, RP) company disclosure: ~1.2M passengers + ~600k vehicles carried in 2017 (+20% over 2016) across Donsak-Lipa Noi (Samui) and Donsak-Phangan routes; ~14 ferries, up to 50 trips/day (RP business plan via Koh Samui News/Samui Times; CreditRiskMonitor profile). RP FY2024 (2567) one-report exists but is a scanned PDF; per-route pax not machine-readable.</t>
+          <t>Koh Samui (Bangrak/Maenam) -&gt; Koh Phangan (Thong Sala)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="29" t="inlineStr">
         <is>
-          <t>Koh Samui</t>
+          <t>Royal_Coast</t>
         </is>
       </c>
       <c r="B11" s="29" t="inlineStr">
@@ -3595,19 +3615,23 @@
       </c>
       <c r="C11" s="30" t="inlineStr">
         <is>
-          <t>Four Seasons Koh Samui (Laem Yai) → Ang Thong Marine Park (Wua Talap)</t>
+          <t>Hua Hin (pier) → Cha-Am (pier)</t>
         </is>
       </c>
       <c r="D11" s="31" t="n">
-        <v>15.3</v>
+        <v>13.4</v>
       </c>
       <c r="E11" s="26" t="n">
-        <v>79</v>
-      </c>
-      <c r="F11" s="32" t="n"/>
+        <v>24</v>
+      </c>
+      <c r="F11" s="32" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
       <c r="G11" s="32" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>low-med</t>
         </is>
       </c>
       <c r="H11" s="19" t="n">
@@ -3710,20 +3734,20 @@
         <v/>
       </c>
       <c r="AG11" s="31" t="n">
-        <v>300000</v>
+        <v>28000</v>
       </c>
       <c r="AH11" s="32" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="AI11" s="32" t="inlineStr">
         <is>
-          <t>med-low</t>
+          <t>low-med</t>
         </is>
       </c>
       <c r="AJ11" s="39" t="n">
-        <v>0.9</v>
+        <v>0.1</v>
       </c>
       <c r="AK11" s="34">
         <f>IF(AG11="","",AG11*AJ11)</f>
@@ -3753,9 +3777,7 @@
       </c>
       <c r="AR11" s="41" t="n"/>
       <c r="AS11" s="41" t="n"/>
-      <c r="AT11" s="42" t="n">
-        <v>3</v>
-      </c>
+      <c r="AT11" s="42" t="n"/>
       <c r="AU11" s="43">
         <f>IF(((S11*pax_cap*load_thin*ROUND(K11*L11*revleg_thin,0))-(((battery/range_nm)*D11*ROUND(K11*L11*revleg_thin,0)*VLOOKUP(B11,country_opex,3,FALSE))+V11+W11+X11+Y11+Z11))&lt;=0,"",VLOOKUP(B11,country_opex,7,FALSE)/((S11*pax_cap*load_thin*ROUND(K11*L11*revleg_thin,0))-(((battery/range_nm)*D11*ROUND(K11*L11*revleg_thin,0)*VLOOKUP(B11,country_opex,3,FALSE))+V11+W11+X11+Y11+Z11)))</f>
         <v/>
@@ -3768,17 +3790,21 @@
         <f>IF(((S11*pax_cap*load_full*ROUND(K11*L11*revleg_full,0))-(((battery/range_nm)*D11*ROUND(K11*L11*revleg_full,0)*VLOOKUP(B11,country_opex,3,FALSE))+V11+W11+X11+Y11+Z11))&lt;=0,"",VLOOKUP(B11,country_opex,7,FALSE)/((S11*pax_cap*load_full*ROUND(K11*L11*revleg_full,0))-(((battery/range_nm)*D11*ROUND(K11*L11*revleg_full,0)*VLOOKUP(B11,country_opex,3,FALSE))+V11+W11+X11+Y11+Z11)))</f>
         <v/>
       </c>
-      <c r="AX11" s="44" t="n"/>
+      <c r="AX11" s="44" t="inlineStr">
+        <is>
+          <t>Royal-coast resort weekend hop; modeled premium slice.</t>
+        </is>
+      </c>
       <c r="AY11" s="44" t="inlineStr">
         <is>
-          <t>Mu Ko Ang Thong National Marine Park: ~160,000 park visitors/yr, ~85% foreign, &gt;THB 40M annual fee revenue (Thai PBS citing park authority, ~2024; DNP visitor-stats system catalog.dnp.go.th is the underlying register - R3-GOLD park-authority class). Park is boat-only and closed annually 1 Nov-15 Dec. Licensed speedboat day tours depart Samui (and Phangan) daily in season.</t>
+          <t>Royal-coast resort weekend hop; modeled premium slice.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="29" t="inlineStr">
         <is>
-          <t>Koh Samui</t>
+          <t>Phuket</t>
         </is>
       </c>
       <c r="B12" s="29" t="inlineStr">
@@ -3788,19 +3814,23 @@
       </c>
       <c r="C12" s="30" t="inlineStr">
         <is>
-          <t>Koh Samui (Nathon) → Donsak (Seatran harbour)</t>
+          <t>Ao Po Pier (Ao Po / Ao Por, NE Phuket) → Khao Phing Kan (James Bond Island), Phang Nga Bay</t>
         </is>
       </c>
       <c r="D12" s="31" t="n">
-        <v>17.9</v>
+        <v>13.5</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>15.2</v>
-      </c>
-      <c r="F12" s="32" t="n"/>
+        <v>90</v>
+      </c>
+      <c r="F12" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
       <c r="G12" s="32" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>med</t>
         </is>
       </c>
       <c r="H12" s="19" t="n">
@@ -3815,7 +3845,7 @@
         <v/>
       </c>
       <c r="K12" s="34">
-        <f>MIN(24,FLOOR(60*service_hr/J12,1))</f>
+        <f>MIN(15,FLOOR(60*service_hr/J12,1))</f>
         <v/>
       </c>
       <c r="L12" s="34">
@@ -3903,18 +3933,10 @@
         <v/>
       </c>
       <c r="AG12" s="31" t="n">
-        <v>666667</v>
-      </c>
-      <c r="AH12" s="32" t="inlineStr">
-        <is>
-          <t>T5</t>
-        </is>
-      </c>
-      <c r="AI12" s="32" t="inlineStr">
-        <is>
-          <t>low-med</t>
-        </is>
-      </c>
+        <v>20000</v>
+      </c>
+      <c r="AH12" s="32" t="n"/>
+      <c r="AI12" s="32" t="n"/>
       <c r="AJ12" s="39" t="n">
         <v>0.1</v>
       </c>
@@ -3959,17 +3981,17 @@
         <f>IF(((S12*pax_cap*load_full*ROUND(K12*L12*revleg_full,0))-(((battery/range_nm)*D12*ROUND(K12*L12*revleg_full,0)*VLOOKUP(B12,country_opex,3,FALSE))+V12+W12+X12+Y12+Z12))&lt;=0,"",VLOOKUP(B12,country_opex,7,FALSE)/((S12*pax_cap*load_full*ROUND(K12*L12*revleg_full,0))-(((battery/range_nm)*D12*ROUND(K12*L12*revleg_full,0)*VLOOKUP(B12,country_opex,3,FALSE))+V12+W12+X12+Y12+Z12)))</f>
         <v/>
       </c>
-      <c r="AX12" s="44" t="n"/>
-      <c r="AY12" s="44" t="inlineStr">
-        <is>
-          <t>SUBSET of rn-347c44e1d360 (do not sum). Seatran Ferry: 6 vessels, ~hourly departures 05:00-19:00 each way, 13-16 kt, ~1.5h crossing, ~450-pax + ~70-car capacity per vessel (Tripadvisor operator page; thailandboattickets.com; C9 Hotelworks cited in city brief). No published Seatran annual ridership found.</t>
-        </is>
-      </c>
+      <c r="AX12" s="44" t="inlineStr">
+        <is>
+          <t>John Gray's Hong by Starlight 3,350 THB/pax agent rate (phukettoursdirect.com/hong-by-starlight.html) / USD 108.89 retail (Agoda activities listing); Phuket Sail Tours sunset/day band 2,200-2,800 THB (phuketexpatguide.com operator comparison, 2026); Simba Sea Trips premium small-group products (TripAdvisor-listed, 18-adult cap, award-positioned above mass market). Anchor = conservative mid of the 2,500-3,900 THB premium band ~ USD 90.</t>
+        </is>
+      </c>
+      <c r="AY12" s="44" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="29" t="inlineStr">
         <is>
-          <t>Phuket</t>
+          <t>Koh Samui</t>
         </is>
       </c>
       <c r="B13" s="29" t="inlineStr">
@@ -3979,23 +4001,19 @@
       </c>
       <c r="C13" s="30" t="inlineStr">
         <is>
-          <t>Phuket (Royal Phuket Marina) → Phang Nga Bay / James Bond Island</t>
+          <t>Koh Samui (Lipa Noi) → Donsak (Raja Ferry pier)</t>
         </is>
       </c>
       <c r="D13" s="31" t="n">
-        <v>20</v>
+        <v>14.3</v>
       </c>
       <c r="E13" s="26" t="n">
-        <v>72</v>
-      </c>
-      <c r="F13" s="32" t="inlineStr">
+        <v>15.2</v>
+      </c>
+      <c r="F13" s="32" t="n"/>
+      <c r="G13" s="32" t="inlineStr">
         <is>
           <t>T3</t>
-        </is>
-      </c>
-      <c r="G13" s="32" t="inlineStr">
-        <is>
-          <t>med</t>
         </is>
       </c>
       <c r="H13" s="19" t="n">
@@ -4010,7 +4028,7 @@
         <v/>
       </c>
       <c r="K13" s="34">
-        <f>MIN(15,FLOOR(60*service_hr/J13,1))</f>
+        <f>MIN(24,FLOOR(60*service_hr/J13,1))</f>
         <v/>
       </c>
       <c r="L13" s="34">
@@ -4098,7 +4116,7 @@
         <v/>
       </c>
       <c r="AG13" s="31" t="n">
-        <v>580000</v>
+        <v>666667</v>
       </c>
       <c r="AH13" s="32" t="inlineStr">
         <is>
@@ -4107,7 +4125,7 @@
       </c>
       <c r="AI13" s="32" t="inlineStr">
         <is>
-          <t>med</t>
+          <t>med-low</t>
         </is>
       </c>
       <c r="AJ13" s="39" t="n">
@@ -4154,21 +4172,17 @@
         <f>IF(((S13*pax_cap*load_full*ROUND(K13*L13*revleg_full,0))-(((battery/range_nm)*D13*ROUND(K13*L13*revleg_full,0)*VLOOKUP(B13,country_opex,3,FALSE))+V13+W13+X13+Y13+Z13))&lt;=0,"",VLOOKUP(B13,country_opex,7,FALSE)/((S13*pax_cap*load_full*ROUND(K13*L13*revleg_full,0))-(((battery/range_nm)*D13*ROUND(K13*L13*revleg_full,0)*VLOOKUP(B13,country_opex,3,FALSE))+V13+W13+X13+Y13+Z13)))</f>
         <v/>
       </c>
-      <c r="AX13" s="44" t="inlineStr">
-        <is>
-          <t>Phuket-&gt;Phang Nga Bay/James Bond Island speedboat day-tour ladder (THB/USD 36): budget longtail ~1,400 THB ($39, phukettoursdirect); standard shared speedboat ~2,500 THB ($69); PREMIUM shared speedboat ~2,600-3,700 THB ($72-103, phiphitours/mythailandtours '$55 low-season' to ~3,700 quoted); private charter speedboat ~29,000-40,900 THB/boat/day (yacht-rental-phuket, phuketdreamcompany) = whole-boat, excluded as overclaim. Premium per-seat anchored ~2,600 THB net of 400 THB park fee = $72.</t>
-        </is>
-      </c>
+      <c r="AX13" s="44" t="n"/>
       <c r="AY13" s="44" t="inlineStr">
         <is>
-          <t>Ao Phang Nga National Park visitors FY2567 (Oct-2023..Sep-2024) = 530,204 (DNP top-10 ranking, #7 by visitors; reported by Prachachat, https://www.prachachat.net/hilight-prachachat/news-1796245, Apr-2025). Park is reachable ONLY by tour boat/longtail/speedboat (no road/air to Khao Phing Kan/Ko Tapu) -&gt; R3-EXCEPTION holds: park arrivals = crossing ridership. DNP also runs e-ticketing at this park (one of 6 pilot parks). Pre-covid FY2019 was ~1M+ (payload note), so FY2024 is the conservative post-covid actual.</t>
+          <t>SUBSET of rn-347c44e1d360 (do not sum). Raja Ferry Port (SET-listed, RP) company disclosure: ~1.2M passengers + ~600k vehicles carried in 2017 (+20% over 2016) across Donsak-Lipa Noi (Samui) and Donsak-Phangan routes; ~14 ferries, up to 50 trips/day (RP business plan via Koh Samui News/Samui Times; CreditRiskMonitor profile). RP FY2024 (2567) one-report exists but is a scanned PDF; per-route pax not machine-readable.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="29" t="inlineStr">
         <is>
-          <t>Phuket</t>
+          <t>Koh Samui</t>
         </is>
       </c>
       <c r="B14" s="29" t="inlineStr">
@@ -4178,19 +4192,19 @@
       </c>
       <c r="C14" s="30" t="inlineStr">
         <is>
-          <t>Phuket → Phi Phi (Tonsai)</t>
+          <t>Four Seasons Koh Samui (Laem Yai) → Ang Thong Marine Park (Wua Talap)</t>
         </is>
       </c>
       <c r="D14" s="31" t="n">
-        <v>25</v>
+        <v>15.3</v>
       </c>
       <c r="E14" s="26" t="n">
-        <v>17.14</v>
+        <v>79</v>
       </c>
       <c r="F14" s="32" t="n"/>
       <c r="G14" s="32" t="inlineStr">
         <is>
-          <t>derived_pending_validation</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="H14" s="19" t="n">
@@ -4293,16 +4307,20 @@
         <v/>
       </c>
       <c r="AG14" s="31" t="n">
-        <v>98124</v>
-      </c>
-      <c r="AH14" s="32" t="n"/>
+        <v>300000</v>
+      </c>
+      <c r="AH14" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
       <c r="AI14" s="32" t="inlineStr">
         <is>
-          <t>derived_pending_validation</t>
+          <t>med-low</t>
         </is>
       </c>
       <c r="AJ14" s="39" t="n">
-        <v>0.1</v>
+        <v>0.9</v>
       </c>
       <c r="AK14" s="34">
         <f>IF(AG14="","",AG14*AJ14)</f>
@@ -4332,7 +4350,9 @@
       </c>
       <c r="AR14" s="41" t="n"/>
       <c r="AS14" s="41" t="n"/>
-      <c r="AT14" s="42" t="n"/>
+      <c r="AT14" s="42" t="n">
+        <v>3</v>
+      </c>
       <c r="AU14" s="43">
         <f>IF(((S14*pax_cap*load_thin*ROUND(K14*L14*revleg_thin,0))-(((battery/range_nm)*D14*ROUND(K14*L14*revleg_thin,0)*VLOOKUP(B14,country_opex,3,FALSE))+V14+W14+X14+Y14+Z14))&lt;=0,"",VLOOKUP(B14,country_opex,7,FALSE)/((S14*pax_cap*load_thin*ROUND(K14*L14*revleg_thin,0))-(((battery/range_nm)*D14*ROUND(K14*L14*revleg_thin,0)*VLOOKUP(B14,country_opex,3,FALSE))+V14+W14+X14+Y14+Z14)))</f>
         <v/>
@@ -4345,21 +4365,17 @@
         <f>IF(((S14*pax_cap*load_full*ROUND(K14*L14*revleg_full,0))-(((battery/range_nm)*D14*ROUND(K14*L14*revleg_full,0)*VLOOKUP(B14,country_opex,3,FALSE))+V14+W14+X14+Y14+Z14))&lt;=0,"",VLOOKUP(B14,country_opex,7,FALSE)/((S14*pax_cap*load_full*ROUND(K14*L14*revleg_full,0))-(((battery/range_nm)*D14*ROUND(K14*L14*revleg_full,0)*VLOOKUP(B14,country_opex,3,FALSE))+V14+W14+X14+Y14+Z14)))</f>
         <v/>
       </c>
-      <c r="AX14" s="44" t="inlineStr">
-        <is>
-          <t>Phuket (Rassada Pier) -&gt; Koh Phi Phi (Tonsai)</t>
-        </is>
-      </c>
+      <c r="AX14" s="44" t="n"/>
       <c r="AY14" s="44" t="inlineStr">
         <is>
-          <t>Phuket (Rassada Pier) -&gt; Koh Phi Phi (Tonsai)</t>
+          <t>Mu Ko Ang Thong National Marine Park: ~160,000 park visitors/yr, ~85% foreign, &gt;THB 40M annual fee revenue (Thai PBS citing park authority, ~2024; DNP visitor-stats system catalog.dnp.go.th is the underlying register - R3-GOLD park-authority class). Park is boat-only and closed annually 1 Nov-15 Dec. Licensed speedboat day tours depart Samui (and Phangan) daily in season.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="29" t="inlineStr">
         <is>
-          <t>Koh Samui</t>
+          <t>Phuket</t>
         </is>
       </c>
       <c r="B15" s="29" t="inlineStr">
@@ -4369,19 +4385,23 @@
       </c>
       <c r="C15" s="30" t="inlineStr">
         <is>
-          <t>Koh Samui (Bangrak) → Don Sak Ferry Harbour</t>
+          <t>Rassada Pier (Phuket Deep Sea Port) → Manoh Pier (Koh Yao Yai)</t>
         </is>
       </c>
       <c r="D15" s="31" t="n">
-        <v>28.1</v>
+        <v>16.9</v>
       </c>
       <c r="E15" s="26" t="n">
-        <v>15.2</v>
-      </c>
-      <c r="F15" s="32" t="n"/>
+        <v>100</v>
+      </c>
+      <c r="F15" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
       <c r="G15" s="32" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>med</t>
         </is>
       </c>
       <c r="H15" s="19" t="n">
@@ -4396,7 +4416,7 @@
         <v/>
       </c>
       <c r="K15" s="34">
-        <f>MIN(24,FLOOR(60*service_hr/J15,1))</f>
+        <f>MIN(15,FLOOR(60*service_hr/J15,1))</f>
         <v/>
       </c>
       <c r="L15" s="34">
@@ -4484,20 +4504,20 @@
         <v/>
       </c>
       <c r="AG15" s="31" t="n">
-        <v>666667</v>
+        <v>8500</v>
       </c>
       <c r="AH15" s="32" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="AI15" s="32" t="inlineStr">
         <is>
-          <t>med-low</t>
+          <t>med</t>
         </is>
       </c>
       <c r="AJ15" s="39" t="n">
-        <v>0.1</v>
+        <v>0.9</v>
       </c>
       <c r="AK15" s="34">
         <f>IF(AG15="","",AG15*AJ15)</f>
@@ -4540,17 +4560,21 @@
         <f>IF(((S15*pax_cap*load_full*ROUND(K15*L15*revleg_full,0))-(((battery/range_nm)*D15*ROUND(K15*L15*revleg_full,0)*VLOOKUP(B15,country_opex,3,FALSE))+V15+W15+X15+Y15+Z15))&lt;=0,"",VLOOKUP(B15,country_opex,7,FALSE)/((S15*pax_cap*load_full*ROUND(K15*L15*revleg_full,0))-(((battery/range_nm)*D15*ROUND(K15*L15*revleg_full,0)*VLOOKUP(B15,country_opex,3,FALSE))+V15+W15+X15+Y15+Z15)))</f>
         <v/>
       </c>
-      <c r="AX15" s="44" t="n"/>
+      <c r="AX15" s="44" t="inlineStr">
+        <is>
+          <t>Minor Hotels captive gateway — Anantara Koh Yao Yai boat-only transfer from Phuket.</t>
+        </is>
+      </c>
       <c r="AY15" s="44" t="inlineStr">
         <is>
-          <t>Total Samui&lt;-&gt;Donsak crossing (all operators/piers). Raja Ferry Port (SET: RP) disclosed ~1.2M passengers carried in 2017 (+20% YoY) across its Donsak-Samui(Lipa Noi)/Donsak-Phangan network, with a 1.5M target (Samui Times / Koh Samui News quoting RP business plan; RP IPO-era disclosure ~600k/yr 2014, Nation Thailand). Seatran runs 6 vessels ~hourly 05:00-19:00 Nathon&lt;-&gt;Donsak (Tripadvisor/operator). Mode balance: Samui drew ~3.54M tourists 2023 (Forbes/C9) vs ~1.4M airport arrivals (Samui Airport 2.8M total pax 2024, BAREIT one-report 56-1) - the majority of non-air arrivals cross at Donsak.</t>
+          <t>minor-hotels-phuket-flagship-economics-DRAFT.json — Koh Yao Yai captive transfer pool</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="29" t="inlineStr">
         <is>
-          <t>Koh Samui</t>
+          <t>Phuket</t>
         </is>
       </c>
       <c r="B16" s="29" t="inlineStr">
@@ -4560,19 +4584,23 @@
       </c>
       <c r="C16" s="30" t="inlineStr">
         <is>
-          <t>Koh Samui → Koh Tao (Mae Haad)</t>
+          <t>Ko Lanta (Saladan Pier) → Koh Phi Phi (Tonsai)</t>
         </is>
       </c>
       <c r="D16" s="31" t="n">
-        <v>35.3</v>
+        <v>17</v>
       </c>
       <c r="E16" s="26" t="n">
-        <v>24.4</v>
-      </c>
-      <c r="F16" s="32" t="n"/>
+        <v>28</v>
+      </c>
+      <c r="F16" s="32" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
       <c r="G16" s="32" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>low-med</t>
         </is>
       </c>
       <c r="H16" s="19" t="n">
@@ -4675,16 +4703,16 @@
         <v/>
       </c>
       <c r="AG16" s="31" t="n">
-        <v>400000</v>
+        <v>62000</v>
       </c>
       <c r="AH16" s="32" t="inlineStr">
         <is>
-          <t>T5</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="AI16" s="32" t="inlineStr">
         <is>
-          <t>med-low</t>
+          <t>low-med</t>
         </is>
       </c>
       <c r="AJ16" s="39" t="n">
@@ -4731,17 +4759,21 @@
         <f>IF(((S16*pax_cap*load_full*ROUND(K16*L16*revleg_full,0))-(((battery/range_nm)*D16*ROUND(K16*L16*revleg_full,0)*VLOOKUP(B16,country_opex,3,FALSE))+V16+W16+X16+Y16+Z16))&lt;=0,"",VLOOKUP(B16,country_opex,7,FALSE)/((S16*pax_cap*load_full*ROUND(K16*L16*revleg_full,0))-(((battery/range_nm)*D16*ROUND(K16*L16*revleg_full,0)*VLOOKUP(B16,country_opex,3,FALSE))+V16+W16+X16+Y16+Z16)))</f>
         <v/>
       </c>
-      <c r="AX16" s="44" t="n"/>
+      <c r="AX16" s="44" t="inlineStr">
+        <is>
+          <t>MODELED premium foiling fare</t>
+        </is>
+      </c>
       <c r="AY16" s="44" t="inlineStr">
         <is>
-          <t>Koh Tao: 666,778 visitors in 2024 (above pre-Covid; record), 327,000 Jan-May 2025, full-year 2025 forecast &gt;700,000 - Koh Tao Tourism Association / TAT figures via Thairath &amp; Daily News (T2 base). Koh Tao is boat-only (no airport, R3-EXCEPTION: arrivals = crossing ridership). Access splits between the Chumphon side (Bangkok route) and the Samui/Phangan side.</t>
+          <t>MODELED tier demand</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="29" t="inlineStr">
         <is>
-          <t>Phuket</t>
+          <t>Koh Samui</t>
         </is>
       </c>
       <c r="B17" s="29" t="inlineStr">
@@ -4751,23 +4783,19 @@
       </c>
       <c r="C17" s="30" t="inlineStr">
         <is>
-          <t>Phuket → Krabi (Ao Nang)</t>
+          <t>Koh Samui (Nathon) → Donsak (Seatran harbour)</t>
         </is>
       </c>
       <c r="D17" s="31" t="n">
-        <v>40</v>
+        <v>17.9</v>
       </c>
       <c r="E17" s="26" t="n">
-        <v>44</v>
-      </c>
-      <c r="F17" s="32" t="inlineStr">
+        <v>15.2</v>
+      </c>
+      <c r="F17" s="32" t="n"/>
+      <c r="G17" s="32" t="inlineStr">
         <is>
           <t>T3</t>
-        </is>
-      </c>
-      <c r="G17" s="32" t="inlineStr">
-        <is>
-          <t>med</t>
         </is>
       </c>
       <c r="H17" s="19" t="n">
@@ -4782,7 +4810,7 @@
         <v/>
       </c>
       <c r="K17" s="34">
-        <f>MIN(15,FLOOR(60*service_hr/J17,1))</f>
+        <f>MIN(24,FLOOR(60*service_hr/J17,1))</f>
         <v/>
       </c>
       <c r="L17" s="34">
@@ -4869,9 +4897,19 @@
         <f>((D17*O17/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D17*O17*VLOOKUP(B17,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG17" s="31" t="n"/>
-      <c r="AH17" s="32" t="n"/>
-      <c r="AI17" s="32" t="n"/>
+      <c r="AG17" s="31" t="n">
+        <v>666667</v>
+      </c>
+      <c r="AH17" s="32" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
+      <c r="AI17" s="32" t="inlineStr">
+        <is>
+          <t>low-med</t>
+        </is>
+      </c>
       <c r="AJ17" s="39" t="n">
         <v>0.1</v>
       </c>
@@ -4898,7 +4936,7 @@
       <c r="AP17" s="40" t="n"/>
       <c r="AQ17" s="32" t="inlineStr">
         <is>
-          <t>Estimated</t>
+          <t>Grounded</t>
         </is>
       </c>
       <c r="AR17" s="41" t="n"/>
@@ -4916,14 +4954,10 @@
         <f>IF(((S17*pax_cap*load_full*ROUND(K17*L17*revleg_full,0))-(((battery/range_nm)*D17*ROUND(K17*L17*revleg_full,0)*VLOOKUP(B17,country_opex,3,FALSE))+V17+W17+X17+Y17+Z17))&lt;=0,"",VLOOKUP(B17,country_opex,7,FALSE)/((S17*pax_cap*load_full*ROUND(K17*L17*revleg_full,0))-(((battery/range_nm)*D17*ROUND(K17*L17*revleg_full,0)*VLOOKUP(B17,country_opex,3,FALSE))+V17+W17+X17+Y17+Z17)))</f>
         <v/>
       </c>
-      <c r="AX17" s="44" t="inlineStr">
-        <is>
-          <t>Phuket-&gt;Krabi (Ao Nang) speedboat premium tier ~comparable to Phi Phi route ($44). Krabi-specific demand re-source pending.</t>
-        </is>
-      </c>
+      <c r="AX17" s="44" t="n"/>
       <c r="AY17" s="44" t="inlineStr">
         <is>
-          <t>Phi Phi demand moved to new Phuket-&gt;Phi Phi corridor per Jaideep 2026-06-09. Krabi (Ao Nang) demand to be sourced separately. Until then: estimated via country cascade.</t>
+          <t>SUBSET of rn-347c44e1d360 (do not sum). Seatran Ferry: 6 vessels, ~hourly departures 05:00-19:00 each way, 13-16 kt, ~1.5h crossing, ~450-pax + ~70-car capacity per vessel (Tripadvisor operator page; thailandboattickets.com; C9 Hotelworks cited in city brief). No published Seatran annual ridership found.</t>
         </is>
       </c>
     </row>
@@ -4940,14 +4974,14 @@
       </c>
       <c r="C18" s="30" t="inlineStr">
         <is>
-          <t>Phuket → Similan / Surin Islands</t>
+          <t>Phuket (Royal Phuket Marina) → Phang Nga Bay / James Bond Island</t>
         </is>
       </c>
       <c r="D18" s="31" t="n">
-        <v>55</v>
+        <v>20</v>
       </c>
       <c r="E18" s="26" t="n">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="F18" s="32" t="inlineStr">
         <is>
@@ -5068,7 +5102,7 @@
       </c>
       <c r="AI18" s="32" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>med</t>
         </is>
       </c>
       <c r="AJ18" s="39" t="n">
@@ -5117,192 +5151,2395 @@
       </c>
       <c r="AX18" s="44" t="inlineStr">
         <is>
+          <t>Phuket-&gt;Phang Nga Bay/James Bond Island speedboat day-tour ladder (THB/USD 36): budget longtail ~1,400 THB ($39, phukettoursdirect); standard shared speedboat ~2,500 THB ($69); PREMIUM shared speedboat ~2,600-3,700 THB ($72-103, phiphitours/mythailandtours '$55 low-season' to ~3,700 quoted); private charter speedboat ~29,000-40,900 THB/boat/day (yacht-rental-phuket, phuketdreamcompany) = whole-boat, excluded as overclaim. Premium per-seat anchored ~2,600 THB net of 400 THB park fee = $72.</t>
+        </is>
+      </c>
+      <c r="AY18" s="44" t="inlineStr">
+        <is>
+          <t>Ao Phang Nga National Park visitors FY2567 (Oct-2023..Sep-2024) = 530,204 (DNP top-10 ranking, #7 by visitors; reported by Prachachat, https://www.prachachat.net/hilight-prachachat/news-1796245, Apr-2025). Park is reachable ONLY by tour boat/longtail/speedboat (no road/air to Khao Phing Kan/Ko Tapu) -&gt; R3-EXCEPTION holds: park arrivals = crossing ridership. DNP also runs e-ticketing at this park (one of 6 pilot parks). Pre-covid FY2019 was ~1M+ (payload note), so FY2024 is the conservative post-covid actual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="29" t="inlineStr">
+        <is>
+          <t>Phuket</t>
+        </is>
+      </c>
+      <c r="B19" s="29" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C19" s="30" t="inlineStr">
+        <is>
+          <t>Ko Lanta (Saladan Pier) → Krabi (Klong Jilad)</t>
+        </is>
+      </c>
+      <c r="D19" s="31" t="n">
+        <v>24</v>
+      </c>
+      <c r="E19" s="26" t="n">
+        <v>32</v>
+      </c>
+      <c r="F19" s="32" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
+      <c r="G19" s="32" t="inlineStr">
+        <is>
+          <t>low-med</t>
+        </is>
+      </c>
+      <c r="H19" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="33">
+        <f>60*D19/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J19" s="33">
+        <f>I19+turn_min+dwell_min</f>
+        <v/>
+      </c>
+      <c r="K19" s="34">
+        <f>MIN(15,FLOOR(60*service_hr/J19,1))</f>
+        <v/>
+      </c>
+      <c r="L19" s="34">
+        <f>ROUND(365*mech_uptime*H19,0)</f>
+        <v/>
+      </c>
+      <c r="M19" s="35">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="N19" s="35">
+        <f>revleg_sel</f>
+        <v/>
+      </c>
+      <c r="O19" s="34">
+        <f>ROUND(K19*L19*revleg_sel,0)</f>
+        <v/>
+      </c>
+      <c r="P19" s="36">
+        <f>load_sel</f>
+        <v/>
+      </c>
+      <c r="Q19" s="36">
+        <f>pax_cap*P19</f>
+        <v/>
+      </c>
+      <c r="R19" s="34">
+        <f>Q19*O19</f>
+        <v/>
+      </c>
+      <c r="S19" s="37">
+        <f>E19*discount</f>
+        <v/>
+      </c>
+      <c r="T19" s="38">
+        <f>S19*R19</f>
+        <v/>
+      </c>
+      <c r="U19" s="38">
+        <f>(battery/range_nm)*D19*O19*VLOOKUP(B19,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="V19" s="38">
+        <f>VLOOKUP(B19,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="W19" s="38">
+        <f>VLOOKUP(B19,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="X19" s="38">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Y19" s="38">
+        <f>VLOOKUP(B19,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="Z19" s="38">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AA19" s="38">
+        <f>U19+V19+W19+X19+Y19+Z19</f>
+        <v/>
+      </c>
+      <c r="AB19" s="38">
+        <f>VLOOKUP(B19,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AC19" s="38">
+        <f>T19-AA19</f>
+        <v/>
+      </c>
+      <c r="AD19" s="35">
+        <f>IF(T19=0,"",AC19/T19)</f>
+        <v/>
+      </c>
+      <c r="AE19" s="36">
+        <f>IF(AC19&lt;=0,"",VLOOKUP(B19,country_opex,7,FALSE)/AC19)</f>
+        <v/>
+      </c>
+      <c r="AF19" s="33">
+        <f>((D19*O19/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D19*O19*VLOOKUP(B19,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AG19" s="31" t="n">
+        <v>28000</v>
+      </c>
+      <c r="AH19" s="32" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="AI19" s="32" t="inlineStr">
+        <is>
+          <t>low-med</t>
+        </is>
+      </c>
+      <c r="AJ19" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AK19" s="34">
+        <f>IF(AG19="","",AG19*AJ19)</f>
+        <v/>
+      </c>
+      <c r="AL19" s="34">
+        <f>IF(OR(AG19="",R19=0),"",MIN(IF(AT19="",9.9E+99,AT19),FLOOR(AK19/R19,1)))</f>
+        <v/>
+      </c>
+      <c r="AM19" s="38">
+        <f>IF(AL19="","",AL19*T19)</f>
+        <v/>
+      </c>
+      <c r="AN19" s="36">
+        <f>IF(OR(AG19="",R19=0),"",MIN(IF(AT19="",9.9E+99,AT19),AK19/R19))</f>
+        <v/>
+      </c>
+      <c r="AO19" s="38">
+        <f>IF(AN19="","",AN19*T19)</f>
+        <v/>
+      </c>
+      <c r="AP19" s="40" t="n"/>
+      <c r="AQ19" s="32" t="inlineStr">
+        <is>
+          <t>Grounded</t>
+        </is>
+      </c>
+      <c r="AR19" s="41" t="n"/>
+      <c r="AS19" s="41" t="n"/>
+      <c r="AT19" s="42" t="n"/>
+      <c r="AU19" s="43">
+        <f>IF(((S19*pax_cap*load_thin*ROUND(K19*L19*revleg_thin,0))-(((battery/range_nm)*D19*ROUND(K19*L19*revleg_thin,0)*VLOOKUP(B19,country_opex,3,FALSE))+V19+W19+X19+Y19+Z19))&lt;=0,"",VLOOKUP(B19,country_opex,7,FALSE)/((S19*pax_cap*load_thin*ROUND(K19*L19*revleg_thin,0))-(((battery/range_nm)*D19*ROUND(K19*L19*revleg_thin,0)*VLOOKUP(B19,country_opex,3,FALSE))+V19+W19+X19+Y19+Z19)))</f>
+        <v/>
+      </c>
+      <c r="AV19" s="43">
+        <f>IF(((S19*pax_cap*load_mid*ROUND(K19*L19*revleg_mid,0))-(((battery/range_nm)*D19*ROUND(K19*L19*revleg_mid,0)*VLOOKUP(B19,country_opex,3,FALSE))+V19+W19+X19+Y19+Z19))&lt;=0,"",VLOOKUP(B19,country_opex,7,FALSE)/((S19*pax_cap*load_mid*ROUND(K19*L19*revleg_mid,0))-(((battery/range_nm)*D19*ROUND(K19*L19*revleg_mid,0)*VLOOKUP(B19,country_opex,3,FALSE))+V19+W19+X19+Y19+Z19)))</f>
+        <v/>
+      </c>
+      <c r="AW19" s="43">
+        <f>IF(((S19*pax_cap*load_full*ROUND(K19*L19*revleg_full,0))-(((battery/range_nm)*D19*ROUND(K19*L19*revleg_full,0)*VLOOKUP(B19,country_opex,3,FALSE))+V19+W19+X19+Y19+Z19))&lt;=0,"",VLOOKUP(B19,country_opex,7,FALSE)/((S19*pax_cap*load_full*ROUND(K19*L19*revleg_full,0))-(((battery/range_nm)*D19*ROUND(K19*L19*revleg_full,0)*VLOOKUP(B19,country_opex,3,FALSE))+V19+W19+X19+Y19+Z19)))</f>
+        <v/>
+      </c>
+      <c r="AX19" s="44" t="inlineStr">
+        <is>
+          <t>MODELED premium foiling fare</t>
+        </is>
+      </c>
+      <c r="AY19" s="44" t="inlineStr">
+        <is>
+          <t>MODELED tier demand</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="29" t="inlineStr">
+        <is>
+          <t>Phuket</t>
+        </is>
+      </c>
+      <c r="B20" s="29" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C20" s="30" t="inlineStr">
+        <is>
+          <t>Phuket → Phi Phi (Tonsai)</t>
+        </is>
+      </c>
+      <c r="D20" s="31" t="n">
+        <v>25</v>
+      </c>
+      <c r="E20" s="26" t="n">
+        <v>17.14</v>
+      </c>
+      <c r="F20" s="32" t="n"/>
+      <c r="G20" s="32" t="inlineStr">
+        <is>
+          <t>derived_pending_validation</t>
+        </is>
+      </c>
+      <c r="H20" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="33">
+        <f>60*D20/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J20" s="33">
+        <f>I20+turn_min+dwell_min</f>
+        <v/>
+      </c>
+      <c r="K20" s="34">
+        <f>MIN(15,FLOOR(60*service_hr/J20,1))</f>
+        <v/>
+      </c>
+      <c r="L20" s="34">
+        <f>ROUND(365*mech_uptime*H20,0)</f>
+        <v/>
+      </c>
+      <c r="M20" s="35">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="N20" s="35">
+        <f>revleg_sel</f>
+        <v/>
+      </c>
+      <c r="O20" s="34">
+        <f>ROUND(K20*L20*revleg_sel,0)</f>
+        <v/>
+      </c>
+      <c r="P20" s="36">
+        <f>load_sel</f>
+        <v/>
+      </c>
+      <c r="Q20" s="36">
+        <f>pax_cap*P20</f>
+        <v/>
+      </c>
+      <c r="R20" s="34">
+        <f>Q20*O20</f>
+        <v/>
+      </c>
+      <c r="S20" s="37">
+        <f>E20*discount</f>
+        <v/>
+      </c>
+      <c r="T20" s="38">
+        <f>S20*R20</f>
+        <v/>
+      </c>
+      <c r="U20" s="38">
+        <f>(battery/range_nm)*D20*O20*VLOOKUP(B20,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="V20" s="38">
+        <f>VLOOKUP(B20,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="W20" s="38">
+        <f>VLOOKUP(B20,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="X20" s="38">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Y20" s="38">
+        <f>VLOOKUP(B20,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="Z20" s="38">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AA20" s="38">
+        <f>U20+V20+W20+X20+Y20+Z20</f>
+        <v/>
+      </c>
+      <c r="AB20" s="38">
+        <f>VLOOKUP(B20,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AC20" s="38">
+        <f>T20-AA20</f>
+        <v/>
+      </c>
+      <c r="AD20" s="35">
+        <f>IF(T20=0,"",AC20/T20)</f>
+        <v/>
+      </c>
+      <c r="AE20" s="36">
+        <f>IF(AC20&lt;=0,"",VLOOKUP(B20,country_opex,7,FALSE)/AC20)</f>
+        <v/>
+      </c>
+      <c r="AF20" s="33">
+        <f>((D20*O20/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D20*O20*VLOOKUP(B20,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AG20" s="31" t="n">
+        <v>98124</v>
+      </c>
+      <c r="AH20" s="32" t="n"/>
+      <c r="AI20" s="32" t="inlineStr">
+        <is>
+          <t>derived_pending_validation</t>
+        </is>
+      </c>
+      <c r="AJ20" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AK20" s="34">
+        <f>IF(AG20="","",AG20*AJ20)</f>
+        <v/>
+      </c>
+      <c r="AL20" s="34">
+        <f>IF(OR(AG20="",R20=0),"",MIN(IF(AT20="",9.9E+99,AT20),FLOOR(AK20/R20,1)))</f>
+        <v/>
+      </c>
+      <c r="AM20" s="38">
+        <f>IF(AL20="","",AL20*T20)</f>
+        <v/>
+      </c>
+      <c r="AN20" s="36">
+        <f>IF(OR(AG20="",R20=0),"",MIN(IF(AT20="",9.9E+99,AT20),AK20/R20))</f>
+        <v/>
+      </c>
+      <c r="AO20" s="38">
+        <f>IF(AN20="","",AN20*T20)</f>
+        <v/>
+      </c>
+      <c r="AP20" s="40" t="n"/>
+      <c r="AQ20" s="32" t="inlineStr">
+        <is>
+          <t>Grounded</t>
+        </is>
+      </c>
+      <c r="AR20" s="41" t="n"/>
+      <c r="AS20" s="41" t="n"/>
+      <c r="AT20" s="42" t="n"/>
+      <c r="AU20" s="43">
+        <f>IF(((S20*pax_cap*load_thin*ROUND(K20*L20*revleg_thin,0))-(((battery/range_nm)*D20*ROUND(K20*L20*revleg_thin,0)*VLOOKUP(B20,country_opex,3,FALSE))+V20+W20+X20+Y20+Z20))&lt;=0,"",VLOOKUP(B20,country_opex,7,FALSE)/((S20*pax_cap*load_thin*ROUND(K20*L20*revleg_thin,0))-(((battery/range_nm)*D20*ROUND(K20*L20*revleg_thin,0)*VLOOKUP(B20,country_opex,3,FALSE))+V20+W20+X20+Y20+Z20)))</f>
+        <v/>
+      </c>
+      <c r="AV20" s="43">
+        <f>IF(((S20*pax_cap*load_mid*ROUND(K20*L20*revleg_mid,0))-(((battery/range_nm)*D20*ROUND(K20*L20*revleg_mid,0)*VLOOKUP(B20,country_opex,3,FALSE))+V20+W20+X20+Y20+Z20))&lt;=0,"",VLOOKUP(B20,country_opex,7,FALSE)/((S20*pax_cap*load_mid*ROUND(K20*L20*revleg_mid,0))-(((battery/range_nm)*D20*ROUND(K20*L20*revleg_mid,0)*VLOOKUP(B20,country_opex,3,FALSE))+V20+W20+X20+Y20+Z20)))</f>
+        <v/>
+      </c>
+      <c r="AW20" s="43">
+        <f>IF(((S20*pax_cap*load_full*ROUND(K20*L20*revleg_full,0))-(((battery/range_nm)*D20*ROUND(K20*L20*revleg_full,0)*VLOOKUP(B20,country_opex,3,FALSE))+V20+W20+X20+Y20+Z20))&lt;=0,"",VLOOKUP(B20,country_opex,7,FALSE)/((S20*pax_cap*load_full*ROUND(K20*L20*revleg_full,0))-(((battery/range_nm)*D20*ROUND(K20*L20*revleg_full,0)*VLOOKUP(B20,country_opex,3,FALSE))+V20+W20+X20+Y20+Z20)))</f>
+        <v/>
+      </c>
+      <c r="AX20" s="44" t="inlineStr">
+        <is>
+          <t>Phuket (Rassada Pier) -&gt; Koh Phi Phi (Tonsai)</t>
+        </is>
+      </c>
+      <c r="AY20" s="44" t="inlineStr">
+        <is>
+          <t>Phuket (Rassada Pier) -&gt; Koh Phi Phi (Tonsai)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="29" t="inlineStr">
+        <is>
+          <t>Koh Samui</t>
+        </is>
+      </c>
+      <c r="B21" s="29" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C21" s="30" t="inlineStr">
+        <is>
+          <t>Koh Samui (Bangrak) → Don Sak Ferry Harbour</t>
+        </is>
+      </c>
+      <c r="D21" s="31" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="E21" s="26" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="F21" s="32" t="n"/>
+      <c r="G21" s="32" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="H21" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="33">
+        <f>60*D21/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J21" s="33">
+        <f>I21+turn_min+dwell_min</f>
+        <v/>
+      </c>
+      <c r="K21" s="34">
+        <f>MIN(24,FLOOR(60*service_hr/J21,1))</f>
+        <v/>
+      </c>
+      <c r="L21" s="34">
+        <f>ROUND(365*mech_uptime*H21,0)</f>
+        <v/>
+      </c>
+      <c r="M21" s="35">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="N21" s="35">
+        <f>revleg_sel</f>
+        <v/>
+      </c>
+      <c r="O21" s="34">
+        <f>ROUND(K21*L21*revleg_sel,0)</f>
+        <v/>
+      </c>
+      <c r="P21" s="36">
+        <f>load_sel</f>
+        <v/>
+      </c>
+      <c r="Q21" s="36">
+        <f>pax_cap*P21</f>
+        <v/>
+      </c>
+      <c r="R21" s="34">
+        <f>Q21*O21</f>
+        <v/>
+      </c>
+      <c r="S21" s="37">
+        <f>E21*discount</f>
+        <v/>
+      </c>
+      <c r="T21" s="38">
+        <f>S21*R21</f>
+        <v/>
+      </c>
+      <c r="U21" s="38">
+        <f>(battery/range_nm)*D21*O21*VLOOKUP(B21,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="V21" s="38">
+        <f>VLOOKUP(B21,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="W21" s="38">
+        <f>VLOOKUP(B21,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="X21" s="38">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Y21" s="38">
+        <f>VLOOKUP(B21,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="Z21" s="38">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AA21" s="38">
+        <f>U21+V21+W21+X21+Y21+Z21</f>
+        <v/>
+      </c>
+      <c r="AB21" s="38">
+        <f>VLOOKUP(B21,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AC21" s="38">
+        <f>T21-AA21</f>
+        <v/>
+      </c>
+      <c r="AD21" s="35">
+        <f>IF(T21=0,"",AC21/T21)</f>
+        <v/>
+      </c>
+      <c r="AE21" s="36">
+        <f>IF(AC21&lt;=0,"",VLOOKUP(B21,country_opex,7,FALSE)/AC21)</f>
+        <v/>
+      </c>
+      <c r="AF21" s="33">
+        <f>((D21*O21/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D21*O21*VLOOKUP(B21,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AG21" s="31" t="n">
+        <v>666667</v>
+      </c>
+      <c r="AH21" s="32" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="AI21" s="32" t="inlineStr">
+        <is>
+          <t>med-low</t>
+        </is>
+      </c>
+      <c r="AJ21" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AK21" s="34">
+        <f>IF(AG21="","",AG21*AJ21)</f>
+        <v/>
+      </c>
+      <c r="AL21" s="34">
+        <f>IF(OR(AG21="",R21=0),"",MIN(IF(AT21="",9.9E+99,AT21),FLOOR(AK21/R21,1)))</f>
+        <v/>
+      </c>
+      <c r="AM21" s="38">
+        <f>IF(AL21="","",AL21*T21)</f>
+        <v/>
+      </c>
+      <c r="AN21" s="36">
+        <f>IF(OR(AG21="",R21=0),"",MIN(IF(AT21="",9.9E+99,AT21),AK21/R21))</f>
+        <v/>
+      </c>
+      <c r="AO21" s="38">
+        <f>IF(AN21="","",AN21*T21)</f>
+        <v/>
+      </c>
+      <c r="AP21" s="40" t="n"/>
+      <c r="AQ21" s="32" t="inlineStr">
+        <is>
+          <t>Grounded</t>
+        </is>
+      </c>
+      <c r="AR21" s="41" t="n"/>
+      <c r="AS21" s="41" t="n"/>
+      <c r="AT21" s="42" t="n"/>
+      <c r="AU21" s="43">
+        <f>IF(((S21*pax_cap*load_thin*ROUND(K21*L21*revleg_thin,0))-(((battery/range_nm)*D21*ROUND(K21*L21*revleg_thin,0)*VLOOKUP(B21,country_opex,3,FALSE))+V21+W21+X21+Y21+Z21))&lt;=0,"",VLOOKUP(B21,country_opex,7,FALSE)/((S21*pax_cap*load_thin*ROUND(K21*L21*revleg_thin,0))-(((battery/range_nm)*D21*ROUND(K21*L21*revleg_thin,0)*VLOOKUP(B21,country_opex,3,FALSE))+V21+W21+X21+Y21+Z21)))</f>
+        <v/>
+      </c>
+      <c r="AV21" s="43">
+        <f>IF(((S21*pax_cap*load_mid*ROUND(K21*L21*revleg_mid,0))-(((battery/range_nm)*D21*ROUND(K21*L21*revleg_mid,0)*VLOOKUP(B21,country_opex,3,FALSE))+V21+W21+X21+Y21+Z21))&lt;=0,"",VLOOKUP(B21,country_opex,7,FALSE)/((S21*pax_cap*load_mid*ROUND(K21*L21*revleg_mid,0))-(((battery/range_nm)*D21*ROUND(K21*L21*revleg_mid,0)*VLOOKUP(B21,country_opex,3,FALSE))+V21+W21+X21+Y21+Z21)))</f>
+        <v/>
+      </c>
+      <c r="AW21" s="43">
+        <f>IF(((S21*pax_cap*load_full*ROUND(K21*L21*revleg_full,0))-(((battery/range_nm)*D21*ROUND(K21*L21*revleg_full,0)*VLOOKUP(B21,country_opex,3,FALSE))+V21+W21+X21+Y21+Z21))&lt;=0,"",VLOOKUP(B21,country_opex,7,FALSE)/((S21*pax_cap*load_full*ROUND(K21*L21*revleg_full,0))-(((battery/range_nm)*D21*ROUND(K21*L21*revleg_full,0)*VLOOKUP(B21,country_opex,3,FALSE))+V21+W21+X21+Y21+Z21)))</f>
+        <v/>
+      </c>
+      <c r="AX21" s="44" t="n"/>
+      <c r="AY21" s="44" t="inlineStr">
+        <is>
+          <t>Total Samui&lt;-&gt;Donsak crossing (all operators/piers). Raja Ferry Port (SET: RP) disclosed ~1.2M passengers carried in 2017 (+20% YoY) across its Donsak-Samui(Lipa Noi)/Donsak-Phangan network, with a 1.5M target (Samui Times / Koh Samui News quoting RP business plan; RP IPO-era disclosure ~600k/yr 2014, Nation Thailand). Seatran runs 6 vessels ~hourly 05:00-19:00 Nathon&lt;-&gt;Donsak (Tripadvisor/operator). Mode balance: Samui drew ~3.54M tourists 2023 (Forbes/C9) vs ~1.4M airport arrivals (Samui Airport 2.8M total pax 2024, BAREIT one-report 56-1) - the majority of non-air arrivals cross at Donsak.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="29" t="inlineStr">
+        <is>
+          <t>Koh Samui</t>
+        </is>
+      </c>
+      <c r="B22" s="29" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C22" s="30" t="inlineStr">
+        <is>
+          <t>Koh Samui → Koh Tao (Mae Haad)</t>
+        </is>
+      </c>
+      <c r="D22" s="31" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="E22" s="26" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="F22" s="32" t="n"/>
+      <c r="G22" s="32" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="H22" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="33">
+        <f>60*D22/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J22" s="33">
+        <f>I22+turn_min+dwell_min</f>
+        <v/>
+      </c>
+      <c r="K22" s="34">
+        <f>MIN(15,FLOOR(60*service_hr/J22,1))</f>
+        <v/>
+      </c>
+      <c r="L22" s="34">
+        <f>ROUND(365*mech_uptime*H22,0)</f>
+        <v/>
+      </c>
+      <c r="M22" s="35">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="N22" s="35">
+        <f>revleg_sel</f>
+        <v/>
+      </c>
+      <c r="O22" s="34">
+        <f>ROUND(K22*L22*revleg_sel,0)</f>
+        <v/>
+      </c>
+      <c r="P22" s="36">
+        <f>load_sel</f>
+        <v/>
+      </c>
+      <c r="Q22" s="36">
+        <f>pax_cap*P22</f>
+        <v/>
+      </c>
+      <c r="R22" s="34">
+        <f>Q22*O22</f>
+        <v/>
+      </c>
+      <c r="S22" s="37">
+        <f>E22*discount</f>
+        <v/>
+      </c>
+      <c r="T22" s="38">
+        <f>S22*R22</f>
+        <v/>
+      </c>
+      <c r="U22" s="38">
+        <f>(battery/range_nm)*D22*O22*VLOOKUP(B22,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="V22" s="38">
+        <f>VLOOKUP(B22,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="W22" s="38">
+        <f>VLOOKUP(B22,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="X22" s="38">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Y22" s="38">
+        <f>VLOOKUP(B22,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="Z22" s="38">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AA22" s="38">
+        <f>U22+V22+W22+X22+Y22+Z22</f>
+        <v/>
+      </c>
+      <c r="AB22" s="38">
+        <f>VLOOKUP(B22,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AC22" s="38">
+        <f>T22-AA22</f>
+        <v/>
+      </c>
+      <c r="AD22" s="35">
+        <f>IF(T22=0,"",AC22/T22)</f>
+        <v/>
+      </c>
+      <c r="AE22" s="36">
+        <f>IF(AC22&lt;=0,"",VLOOKUP(B22,country_opex,7,FALSE)/AC22)</f>
+        <v/>
+      </c>
+      <c r="AF22" s="33">
+        <f>((D22*O22/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D22*O22*VLOOKUP(B22,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AG22" s="31" t="n">
+        <v>400000</v>
+      </c>
+      <c r="AH22" s="32" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
+      <c r="AI22" s="32" t="inlineStr">
+        <is>
+          <t>med-low</t>
+        </is>
+      </c>
+      <c r="AJ22" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AK22" s="34">
+        <f>IF(AG22="","",AG22*AJ22)</f>
+        <v/>
+      </c>
+      <c r="AL22" s="34">
+        <f>IF(OR(AG22="",R22=0),"",MIN(IF(AT22="",9.9E+99,AT22),FLOOR(AK22/R22,1)))</f>
+        <v/>
+      </c>
+      <c r="AM22" s="38">
+        <f>IF(AL22="","",AL22*T22)</f>
+        <v/>
+      </c>
+      <c r="AN22" s="36">
+        <f>IF(OR(AG22="",R22=0),"",MIN(IF(AT22="",9.9E+99,AT22),AK22/R22))</f>
+        <v/>
+      </c>
+      <c r="AO22" s="38">
+        <f>IF(AN22="","",AN22*T22)</f>
+        <v/>
+      </c>
+      <c r="AP22" s="40" t="n"/>
+      <c r="AQ22" s="32" t="inlineStr">
+        <is>
+          <t>Grounded</t>
+        </is>
+      </c>
+      <c r="AR22" s="41" t="n"/>
+      <c r="AS22" s="41" t="n"/>
+      <c r="AT22" s="42" t="n"/>
+      <c r="AU22" s="43">
+        <f>IF(((S22*pax_cap*load_thin*ROUND(K22*L22*revleg_thin,0))-(((battery/range_nm)*D22*ROUND(K22*L22*revleg_thin,0)*VLOOKUP(B22,country_opex,3,FALSE))+V22+W22+X22+Y22+Z22))&lt;=0,"",VLOOKUP(B22,country_opex,7,FALSE)/((S22*pax_cap*load_thin*ROUND(K22*L22*revleg_thin,0))-(((battery/range_nm)*D22*ROUND(K22*L22*revleg_thin,0)*VLOOKUP(B22,country_opex,3,FALSE))+V22+W22+X22+Y22+Z22)))</f>
+        <v/>
+      </c>
+      <c r="AV22" s="43">
+        <f>IF(((S22*pax_cap*load_mid*ROUND(K22*L22*revleg_mid,0))-(((battery/range_nm)*D22*ROUND(K22*L22*revleg_mid,0)*VLOOKUP(B22,country_opex,3,FALSE))+V22+W22+X22+Y22+Z22))&lt;=0,"",VLOOKUP(B22,country_opex,7,FALSE)/((S22*pax_cap*load_mid*ROUND(K22*L22*revleg_mid,0))-(((battery/range_nm)*D22*ROUND(K22*L22*revleg_mid,0)*VLOOKUP(B22,country_opex,3,FALSE))+V22+W22+X22+Y22+Z22)))</f>
+        <v/>
+      </c>
+      <c r="AW22" s="43">
+        <f>IF(((S22*pax_cap*load_full*ROUND(K22*L22*revleg_full,0))-(((battery/range_nm)*D22*ROUND(K22*L22*revleg_full,0)*VLOOKUP(B22,country_opex,3,FALSE))+V22+W22+X22+Y22+Z22))&lt;=0,"",VLOOKUP(B22,country_opex,7,FALSE)/((S22*pax_cap*load_full*ROUND(K22*L22*revleg_full,0))-(((battery/range_nm)*D22*ROUND(K22*L22*revleg_full,0)*VLOOKUP(B22,country_opex,3,FALSE))+V22+W22+X22+Y22+Z22)))</f>
+        <v/>
+      </c>
+      <c r="AX22" s="44" t="n"/>
+      <c r="AY22" s="44" t="inlineStr">
+        <is>
+          <t>Koh Tao: 666,778 visitors in 2024 (above pre-Covid; record), 327,000 Jan-May 2025, full-year 2025 forecast &gt;700,000 - Koh Tao Tourism Association / TAT figures via Thairath &amp; Daily News (T2 base). Koh Tao is boat-only (no airport, R3-EXCEPTION: arrivals = crossing ridership). Access splits between the Chumphon side (Bangkok route) and the Samui/Phangan side.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="29" t="inlineStr">
+        <is>
+          <t>Phuket</t>
+        </is>
+      </c>
+      <c r="B23" s="29" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C23" s="30" t="inlineStr">
+        <is>
+          <t>Manoh Pier (Koh Yao Yai) → Thap Lamu Pier (Similan Gateway)</t>
+        </is>
+      </c>
+      <c r="D23" s="31" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="E23" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="F23" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G23" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="H23" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="33">
+        <f>60*D23/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J23" s="33">
+        <f>I23+turn_min+dwell_min</f>
+        <v/>
+      </c>
+      <c r="K23" s="34">
+        <f>MIN(15,FLOOR(60*service_hr/J23,1))</f>
+        <v/>
+      </c>
+      <c r="L23" s="34">
+        <f>ROUND(365*mech_uptime*H23,0)</f>
+        <v/>
+      </c>
+      <c r="M23" s="35">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="N23" s="35">
+        <f>revleg_sel</f>
+        <v/>
+      </c>
+      <c r="O23" s="34">
+        <f>ROUND(K23*L23*revleg_sel,0)</f>
+        <v/>
+      </c>
+      <c r="P23" s="36">
+        <f>load_sel</f>
+        <v/>
+      </c>
+      <c r="Q23" s="36">
+        <f>pax_cap*P23</f>
+        <v/>
+      </c>
+      <c r="R23" s="34">
+        <f>Q23*O23</f>
+        <v/>
+      </c>
+      <c r="S23" s="37">
+        <f>E23*discount</f>
+        <v/>
+      </c>
+      <c r="T23" s="38">
+        <f>S23*R23</f>
+        <v/>
+      </c>
+      <c r="U23" s="38">
+        <f>(battery/range_nm)*D23*O23*VLOOKUP(B23,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="V23" s="38">
+        <f>VLOOKUP(B23,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="W23" s="38">
+        <f>VLOOKUP(B23,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="X23" s="38">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Y23" s="38">
+        <f>VLOOKUP(B23,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="Z23" s="38">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AA23" s="38">
+        <f>U23+V23+W23+X23+Y23+Z23</f>
+        <v/>
+      </c>
+      <c r="AB23" s="38">
+        <f>VLOOKUP(B23,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AC23" s="38">
+        <f>T23-AA23</f>
+        <v/>
+      </c>
+      <c r="AD23" s="35">
+        <f>IF(T23=0,"",AC23/T23)</f>
+        <v/>
+      </c>
+      <c r="AE23" s="36">
+        <f>IF(AC23&lt;=0,"",VLOOKUP(B23,country_opex,7,FALSE)/AC23)</f>
+        <v/>
+      </c>
+      <c r="AF23" s="33">
+        <f>((D23*O23/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D23*O23*VLOOKUP(B23,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AG23" s="31" t="n">
+        <v>8500</v>
+      </c>
+      <c r="AH23" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="AI23" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="AJ23" s="39" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AK23" s="34">
+        <f>IF(AG23="","",AG23*AJ23)</f>
+        <v/>
+      </c>
+      <c r="AL23" s="34">
+        <f>IF(OR(AG23="",R23=0),"",MIN(IF(AT23="",9.9E+99,AT23),FLOOR(AK23/R23,1)))</f>
+        <v/>
+      </c>
+      <c r="AM23" s="38">
+        <f>IF(AL23="","",AL23*T23)</f>
+        <v/>
+      </c>
+      <c r="AN23" s="36">
+        <f>IF(OR(AG23="",R23=0),"",MIN(IF(AT23="",9.9E+99,AT23),AK23/R23))</f>
+        <v/>
+      </c>
+      <c r="AO23" s="38">
+        <f>IF(AN23="","",AN23*T23)</f>
+        <v/>
+      </c>
+      <c r="AP23" s="40" t="n"/>
+      <c r="AQ23" s="32" t="inlineStr">
+        <is>
+          <t>Grounded</t>
+        </is>
+      </c>
+      <c r="AR23" s="41" t="n"/>
+      <c r="AS23" s="41" t="n"/>
+      <c r="AT23" s="42" t="n"/>
+      <c r="AU23" s="43">
+        <f>IF(((S23*pax_cap*load_thin*ROUND(K23*L23*revleg_thin,0))-(((battery/range_nm)*D23*ROUND(K23*L23*revleg_thin,0)*VLOOKUP(B23,country_opex,3,FALSE))+V23+W23+X23+Y23+Z23))&lt;=0,"",VLOOKUP(B23,country_opex,7,FALSE)/((S23*pax_cap*load_thin*ROUND(K23*L23*revleg_thin,0))-(((battery/range_nm)*D23*ROUND(K23*L23*revleg_thin,0)*VLOOKUP(B23,country_opex,3,FALSE))+V23+W23+X23+Y23+Z23)))</f>
+        <v/>
+      </c>
+      <c r="AV23" s="43">
+        <f>IF(((S23*pax_cap*load_mid*ROUND(K23*L23*revleg_mid,0))-(((battery/range_nm)*D23*ROUND(K23*L23*revleg_mid,0)*VLOOKUP(B23,country_opex,3,FALSE))+V23+W23+X23+Y23+Z23))&lt;=0,"",VLOOKUP(B23,country_opex,7,FALSE)/((S23*pax_cap*load_mid*ROUND(K23*L23*revleg_mid,0))-(((battery/range_nm)*D23*ROUND(K23*L23*revleg_mid,0)*VLOOKUP(B23,country_opex,3,FALSE))+V23+W23+X23+Y23+Z23)))</f>
+        <v/>
+      </c>
+      <c r="AW23" s="43">
+        <f>IF(((S23*pax_cap*load_full*ROUND(K23*L23*revleg_full,0))-(((battery/range_nm)*D23*ROUND(K23*L23*revleg_full,0)*VLOOKUP(B23,country_opex,3,FALSE))+V23+W23+X23+Y23+Z23))&lt;=0,"",VLOOKUP(B23,country_opex,7,FALSE)/((S23*pax_cap*load_full*ROUND(K23*L23*revleg_full,0))-(((battery/range_nm)*D23*ROUND(K23*L23*revleg_full,0)*VLOOKUP(B23,country_opex,3,FALSE))+V23+W23+X23+Y23+Z23)))</f>
+        <v/>
+      </c>
+      <c r="AX23" s="44" t="inlineStr">
+        <is>
+          <t>Minor Hotels inter-resort hop — Koh Yao Yai ↔ Khao Lak portfolio.</t>
+        </is>
+      </c>
+      <c r="AY23" s="44" t="inlineStr">
+        <is>
+          <t>minor-hotels-phuket-flagship-economics-DRAFT.json — inter-brand Andaman hop</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="29" t="inlineStr">
+        <is>
+          <t>Eastern_Seaboard</t>
+        </is>
+      </c>
+      <c r="B24" s="29" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C24" s="30" t="inlineStr">
+        <is>
+          <t>Pattaya (Bali Hai Pier) → Koh Samet (Na Dan Pier)</t>
+        </is>
+      </c>
+      <c r="D24" s="31" t="n">
+        <v>37</v>
+      </c>
+      <c r="E24" s="26" t="n">
+        <v>42</v>
+      </c>
+      <c r="F24" s="32" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
+      <c r="G24" s="32" t="inlineStr">
+        <is>
+          <t>low-med</t>
+        </is>
+      </c>
+      <c r="H24" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" s="33">
+        <f>60*D24/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J24" s="33">
+        <f>I24+turn_min+dwell_min</f>
+        <v/>
+      </c>
+      <c r="K24" s="34">
+        <f>MIN(15,FLOOR(60*service_hr/J24,1))</f>
+        <v/>
+      </c>
+      <c r="L24" s="34">
+        <f>ROUND(365*mech_uptime*H24,0)</f>
+        <v/>
+      </c>
+      <c r="M24" s="35">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="N24" s="35">
+        <f>revleg_sel</f>
+        <v/>
+      </c>
+      <c r="O24" s="34">
+        <f>ROUND(K24*L24*revleg_sel,0)</f>
+        <v/>
+      </c>
+      <c r="P24" s="36">
+        <f>load_sel</f>
+        <v/>
+      </c>
+      <c r="Q24" s="36">
+        <f>pax_cap*P24</f>
+        <v/>
+      </c>
+      <c r="R24" s="34">
+        <f>Q24*O24</f>
+        <v/>
+      </c>
+      <c r="S24" s="37">
+        <f>E24*discount</f>
+        <v/>
+      </c>
+      <c r="T24" s="38">
+        <f>S24*R24</f>
+        <v/>
+      </c>
+      <c r="U24" s="38">
+        <f>(battery/range_nm)*D24*O24*VLOOKUP(B24,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="V24" s="38">
+        <f>VLOOKUP(B24,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="W24" s="38">
+        <f>VLOOKUP(B24,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="X24" s="38">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Y24" s="38">
+        <f>VLOOKUP(B24,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="Z24" s="38">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AA24" s="38">
+        <f>U24+V24+W24+X24+Y24+Z24</f>
+        <v/>
+      </c>
+      <c r="AB24" s="38">
+        <f>VLOOKUP(B24,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AC24" s="38">
+        <f>T24-AA24</f>
+        <v/>
+      </c>
+      <c r="AD24" s="35">
+        <f>IF(T24=0,"",AC24/T24)</f>
+        <v/>
+      </c>
+      <c r="AE24" s="36">
+        <f>IF(AC24&lt;=0,"",VLOOKUP(B24,country_opex,7,FALSE)/AC24)</f>
+        <v/>
+      </c>
+      <c r="AF24" s="33">
+        <f>((D24*O24/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D24*O24*VLOOKUP(B24,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AG24" s="31" t="n">
+        <v>28000</v>
+      </c>
+      <c r="AH24" s="32" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="AI24" s="32" t="inlineStr">
+        <is>
+          <t>low-med</t>
+        </is>
+      </c>
+      <c r="AJ24" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AK24" s="34">
+        <f>IF(AG24="","",AG24*AJ24)</f>
+        <v/>
+      </c>
+      <c r="AL24" s="34">
+        <f>IF(OR(AG24="",R24=0),"",MIN(IF(AT24="",9.9E+99,AT24),FLOOR(AK24/R24,1)))</f>
+        <v/>
+      </c>
+      <c r="AM24" s="38">
+        <f>IF(AL24="","",AL24*T24)</f>
+        <v/>
+      </c>
+      <c r="AN24" s="36">
+        <f>IF(OR(AG24="",R24=0),"",MIN(IF(AT24="",9.9E+99,AT24),AK24/R24))</f>
+        <v/>
+      </c>
+      <c r="AO24" s="38">
+        <f>IF(AN24="","",AN24*T24)</f>
+        <v/>
+      </c>
+      <c r="AP24" s="40" t="n"/>
+      <c r="AQ24" s="32" t="inlineStr">
+        <is>
+          <t>Grounded</t>
+        </is>
+      </c>
+      <c r="AR24" s="41" t="n"/>
+      <c r="AS24" s="41" t="n"/>
+      <c r="AT24" s="42" t="n"/>
+      <c r="AU24" s="43">
+        <f>IF(((S24*pax_cap*load_thin*ROUND(K24*L24*revleg_thin,0))-(((battery/range_nm)*D24*ROUND(K24*L24*revleg_thin,0)*VLOOKUP(B24,country_opex,3,FALSE))+V24+W24+X24+Y24+Z24))&lt;=0,"",VLOOKUP(B24,country_opex,7,FALSE)/((S24*pax_cap*load_thin*ROUND(K24*L24*revleg_thin,0))-(((battery/range_nm)*D24*ROUND(K24*L24*revleg_thin,0)*VLOOKUP(B24,country_opex,3,FALSE))+V24+W24+X24+Y24+Z24)))</f>
+        <v/>
+      </c>
+      <c r="AV24" s="43">
+        <f>IF(((S24*pax_cap*load_mid*ROUND(K24*L24*revleg_mid,0))-(((battery/range_nm)*D24*ROUND(K24*L24*revleg_mid,0)*VLOOKUP(B24,country_opex,3,FALSE))+V24+W24+X24+Y24+Z24))&lt;=0,"",VLOOKUP(B24,country_opex,7,FALSE)/((S24*pax_cap*load_mid*ROUND(K24*L24*revleg_mid,0))-(((battery/range_nm)*D24*ROUND(K24*L24*revleg_mid,0)*VLOOKUP(B24,country_opex,3,FALSE))+V24+W24+X24+Y24+Z24)))</f>
+        <v/>
+      </c>
+      <c r="AW24" s="43">
+        <f>IF(((S24*pax_cap*load_full*ROUND(K24*L24*revleg_full,0))-(((battery/range_nm)*D24*ROUND(K24*L24*revleg_full,0)*VLOOKUP(B24,country_opex,3,FALSE))+V24+W24+X24+Y24+Z24))&lt;=0,"",VLOOKUP(B24,country_opex,7,FALSE)/((S24*pax_cap*load_full*ROUND(K24*L24*revleg_full,0))-(((battery/range_nm)*D24*ROUND(K24*L24*revleg_full,0)*VLOOKUP(B24,country_opex,3,FALSE))+V24+W24+X24+Y24+Z24)))</f>
+        <v/>
+      </c>
+      <c r="AX24" s="44" t="inlineStr">
+        <is>
+          <t>Premium slice of Ban Phe-origin Samet day-trip flow rerouted from Pattaya.</t>
+        </is>
+      </c>
+      <c r="AY24" s="44" t="inlineStr">
+        <is>
+          <t>Premium slice of Ban Phe-origin Samet day-trip flow rerouted from Pattaya.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="29" t="inlineStr">
+        <is>
+          <t>Phuket</t>
+        </is>
+      </c>
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C25" s="30" t="inlineStr">
+        <is>
+          <t>Phuket → Krabi (Ao Nang)</t>
+        </is>
+      </c>
+      <c r="D25" s="31" t="n">
+        <v>40</v>
+      </c>
+      <c r="E25" s="26" t="n">
+        <v>44</v>
+      </c>
+      <c r="F25" s="32" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="G25" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="H25" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" s="33">
+        <f>60*D25/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J25" s="33">
+        <f>I25+turn_min+dwell_min</f>
+        <v/>
+      </c>
+      <c r="K25" s="34">
+        <f>MIN(15,FLOOR(60*service_hr/J25,1))</f>
+        <v/>
+      </c>
+      <c r="L25" s="34">
+        <f>ROUND(365*mech_uptime*H25,0)</f>
+        <v/>
+      </c>
+      <c r="M25" s="35">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="N25" s="35">
+        <f>revleg_sel</f>
+        <v/>
+      </c>
+      <c r="O25" s="34">
+        <f>ROUND(K25*L25*revleg_sel,0)</f>
+        <v/>
+      </c>
+      <c r="P25" s="36">
+        <f>load_sel</f>
+        <v/>
+      </c>
+      <c r="Q25" s="36">
+        <f>pax_cap*P25</f>
+        <v/>
+      </c>
+      <c r="R25" s="34">
+        <f>Q25*O25</f>
+        <v/>
+      </c>
+      <c r="S25" s="37">
+        <f>E25*discount</f>
+        <v/>
+      </c>
+      <c r="T25" s="38">
+        <f>S25*R25</f>
+        <v/>
+      </c>
+      <c r="U25" s="38">
+        <f>(battery/range_nm)*D25*O25*VLOOKUP(B25,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="V25" s="38">
+        <f>VLOOKUP(B25,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="W25" s="38">
+        <f>VLOOKUP(B25,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="X25" s="38">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Y25" s="38">
+        <f>VLOOKUP(B25,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="Z25" s="38">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AA25" s="38">
+        <f>U25+V25+W25+X25+Y25+Z25</f>
+        <v/>
+      </c>
+      <c r="AB25" s="38">
+        <f>VLOOKUP(B25,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AC25" s="38">
+        <f>T25-AA25</f>
+        <v/>
+      </c>
+      <c r="AD25" s="35">
+        <f>IF(T25=0,"",AC25/T25)</f>
+        <v/>
+      </c>
+      <c r="AE25" s="36">
+        <f>IF(AC25&lt;=0,"",VLOOKUP(B25,country_opex,7,FALSE)/AC25)</f>
+        <v/>
+      </c>
+      <c r="AF25" s="33">
+        <f>((D25*O25/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D25*O25*VLOOKUP(B25,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AG25" s="31" t="n"/>
+      <c r="AH25" s="32" t="n"/>
+      <c r="AI25" s="32" t="n"/>
+      <c r="AJ25" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AK25" s="34">
+        <f>IF(AG25="","",AG25*AJ25)</f>
+        <v/>
+      </c>
+      <c r="AL25" s="34">
+        <f>IF(OR(AG25="",R25=0),"",MIN(IF(AT25="",9.9E+99,AT25),FLOOR(AK25/R25,1)))</f>
+        <v/>
+      </c>
+      <c r="AM25" s="38">
+        <f>IF(AL25="","",AL25*T25)</f>
+        <v/>
+      </c>
+      <c r="AN25" s="36">
+        <f>IF(OR(AG25="",R25=0),"",MIN(IF(AT25="",9.9E+99,AT25),AK25/R25))</f>
+        <v/>
+      </c>
+      <c r="AO25" s="38">
+        <f>IF(AN25="","",AN25*T25)</f>
+        <v/>
+      </c>
+      <c r="AP25" s="40" t="n"/>
+      <c r="AQ25" s="32" t="inlineStr">
+        <is>
+          <t>Estimated</t>
+        </is>
+      </c>
+      <c r="AR25" s="41" t="n"/>
+      <c r="AS25" s="41" t="n"/>
+      <c r="AT25" s="42" t="n"/>
+      <c r="AU25" s="43">
+        <f>IF(((S25*pax_cap*load_thin*ROUND(K25*L25*revleg_thin,0))-(((battery/range_nm)*D25*ROUND(K25*L25*revleg_thin,0)*VLOOKUP(B25,country_opex,3,FALSE))+V25+W25+X25+Y25+Z25))&lt;=0,"",VLOOKUP(B25,country_opex,7,FALSE)/((S25*pax_cap*load_thin*ROUND(K25*L25*revleg_thin,0))-(((battery/range_nm)*D25*ROUND(K25*L25*revleg_thin,0)*VLOOKUP(B25,country_opex,3,FALSE))+V25+W25+X25+Y25+Z25)))</f>
+        <v/>
+      </c>
+      <c r="AV25" s="43">
+        <f>IF(((S25*pax_cap*load_mid*ROUND(K25*L25*revleg_mid,0))-(((battery/range_nm)*D25*ROUND(K25*L25*revleg_mid,0)*VLOOKUP(B25,country_opex,3,FALSE))+V25+W25+X25+Y25+Z25))&lt;=0,"",VLOOKUP(B25,country_opex,7,FALSE)/((S25*pax_cap*load_mid*ROUND(K25*L25*revleg_mid,0))-(((battery/range_nm)*D25*ROUND(K25*L25*revleg_mid,0)*VLOOKUP(B25,country_opex,3,FALSE))+V25+W25+X25+Y25+Z25)))</f>
+        <v/>
+      </c>
+      <c r="AW25" s="43">
+        <f>IF(((S25*pax_cap*load_full*ROUND(K25*L25*revleg_full,0))-(((battery/range_nm)*D25*ROUND(K25*L25*revleg_full,0)*VLOOKUP(B25,country_opex,3,FALSE))+V25+W25+X25+Y25+Z25))&lt;=0,"",VLOOKUP(B25,country_opex,7,FALSE)/((S25*pax_cap*load_full*ROUND(K25*L25*revleg_full,0))-(((battery/range_nm)*D25*ROUND(K25*L25*revleg_full,0)*VLOOKUP(B25,country_opex,3,FALSE))+V25+W25+X25+Y25+Z25)))</f>
+        <v/>
+      </c>
+      <c r="AX25" s="44" t="inlineStr">
+        <is>
+          <t>Phuket-&gt;Krabi (Ao Nang) speedboat premium tier ~comparable to Phi Phi route ($44). Krabi-specific demand re-source pending.</t>
+        </is>
+      </c>
+      <c r="AY25" s="44" t="inlineStr">
+        <is>
+          <t>Phi Phi demand moved to new Phuket-&gt;Phi Phi corridor per Jaideep 2026-06-09. Krabi (Ao Nang) demand to be sourced separately. Until then: estimated via country cascade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="29" t="inlineStr">
+        <is>
+          <t>Phuket</t>
+        </is>
+      </c>
+      <c r="B26" s="29" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C26" s="30" t="inlineStr">
+        <is>
+          <t>Phuket (Rassada Pier) → Ko Lanta (Saladan Pier)</t>
+        </is>
+      </c>
+      <c r="D26" s="31" t="n">
+        <v>42.4</v>
+      </c>
+      <c r="E26" s="26" t="n">
+        <v>55</v>
+      </c>
+      <c r="F26" s="32" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
+      <c r="G26" s="32" t="inlineStr">
+        <is>
+          <t>low-med</t>
+        </is>
+      </c>
+      <c r="H26" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I26" s="33">
+        <f>60*D26/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J26" s="33">
+        <f>I26+turn_min+dwell_min</f>
+        <v/>
+      </c>
+      <c r="K26" s="34">
+        <f>MIN(15,FLOOR(60*service_hr/J26,1))</f>
+        <v/>
+      </c>
+      <c r="L26" s="34">
+        <f>ROUND(365*mech_uptime*H26,0)</f>
+        <v/>
+      </c>
+      <c r="M26" s="35">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="N26" s="35">
+        <f>revleg_sel</f>
+        <v/>
+      </c>
+      <c r="O26" s="34">
+        <f>ROUND(K26*L26*revleg_sel,0)</f>
+        <v/>
+      </c>
+      <c r="P26" s="36">
+        <f>load_sel</f>
+        <v/>
+      </c>
+      <c r="Q26" s="36">
+        <f>pax_cap*P26</f>
+        <v/>
+      </c>
+      <c r="R26" s="34">
+        <f>Q26*O26</f>
+        <v/>
+      </c>
+      <c r="S26" s="37">
+        <f>E26*discount</f>
+        <v/>
+      </c>
+      <c r="T26" s="38">
+        <f>S26*R26</f>
+        <v/>
+      </c>
+      <c r="U26" s="38">
+        <f>(battery/range_nm)*D26*O26*VLOOKUP(B26,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="V26" s="38">
+        <f>VLOOKUP(B26,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="W26" s="38">
+        <f>VLOOKUP(B26,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="X26" s="38">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Y26" s="38">
+        <f>VLOOKUP(B26,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="Z26" s="38">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AA26" s="38">
+        <f>U26+V26+W26+X26+Y26+Z26</f>
+        <v/>
+      </c>
+      <c r="AB26" s="38">
+        <f>VLOOKUP(B26,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AC26" s="38">
+        <f>T26-AA26</f>
+        <v/>
+      </c>
+      <c r="AD26" s="35">
+        <f>IF(T26=0,"",AC26/T26)</f>
+        <v/>
+      </c>
+      <c r="AE26" s="36">
+        <f>IF(AC26&lt;=0,"",VLOOKUP(B26,country_opex,7,FALSE)/AC26)</f>
+        <v/>
+      </c>
+      <c r="AF26" s="33">
+        <f>((D26*O26/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D26*O26*VLOOKUP(B26,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AG26" s="31" t="n">
+        <v>31000</v>
+      </c>
+      <c r="AH26" s="32" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="AI26" s="32" t="inlineStr">
+        <is>
+          <t>low-med</t>
+        </is>
+      </c>
+      <c r="AJ26" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AK26" s="34">
+        <f>IF(AG26="","",AG26*AJ26)</f>
+        <v/>
+      </c>
+      <c r="AL26" s="34">
+        <f>IF(OR(AG26="",R26=0),"",MIN(IF(AT26="",9.9E+99,AT26),FLOOR(AK26/R26,1)))</f>
+        <v/>
+      </c>
+      <c r="AM26" s="38">
+        <f>IF(AL26="","",AL26*T26)</f>
+        <v/>
+      </c>
+      <c r="AN26" s="36">
+        <f>IF(OR(AG26="",R26=0),"",MIN(IF(AT26="",9.9E+99,AT26),AK26/R26))</f>
+        <v/>
+      </c>
+      <c r="AO26" s="38">
+        <f>IF(AN26="","",AN26*T26)</f>
+        <v/>
+      </c>
+      <c r="AP26" s="40" t="n"/>
+      <c r="AQ26" s="32" t="inlineStr">
+        <is>
+          <t>Grounded</t>
+        </is>
+      </c>
+      <c r="AR26" s="41" t="n"/>
+      <c r="AS26" s="41" t="n"/>
+      <c r="AT26" s="42" t="n"/>
+      <c r="AU26" s="43">
+        <f>IF(((S26*pax_cap*load_thin*ROUND(K26*L26*revleg_thin,0))-(((battery/range_nm)*D26*ROUND(K26*L26*revleg_thin,0)*VLOOKUP(B26,country_opex,3,FALSE))+V26+W26+X26+Y26+Z26))&lt;=0,"",VLOOKUP(B26,country_opex,7,FALSE)/((S26*pax_cap*load_thin*ROUND(K26*L26*revleg_thin,0))-(((battery/range_nm)*D26*ROUND(K26*L26*revleg_thin,0)*VLOOKUP(B26,country_opex,3,FALSE))+V26+W26+X26+Y26+Z26)))</f>
+        <v/>
+      </c>
+      <c r="AV26" s="43">
+        <f>IF(((S26*pax_cap*load_mid*ROUND(K26*L26*revleg_mid,0))-(((battery/range_nm)*D26*ROUND(K26*L26*revleg_mid,0)*VLOOKUP(B26,country_opex,3,FALSE))+V26+W26+X26+Y26+Z26))&lt;=0,"",VLOOKUP(B26,country_opex,7,FALSE)/((S26*pax_cap*load_mid*ROUND(K26*L26*revleg_mid,0))-(((battery/range_nm)*D26*ROUND(K26*L26*revleg_mid,0)*VLOOKUP(B26,country_opex,3,FALSE))+V26+W26+X26+Y26+Z26)))</f>
+        <v/>
+      </c>
+      <c r="AW26" s="43">
+        <f>IF(((S26*pax_cap*load_full*ROUND(K26*L26*revleg_full,0))-(((battery/range_nm)*D26*ROUND(K26*L26*revleg_full,0)*VLOOKUP(B26,country_opex,3,FALSE))+V26+W26+X26+Y26+Z26))&lt;=0,"",VLOOKUP(B26,country_opex,7,FALSE)/((S26*pax_cap*load_full*ROUND(K26*L26*revleg_full,0))-(((battery/range_nm)*D26*ROUND(K26*L26*revleg_full,0)*VLOOKUP(B26,country_opex,3,FALSE))+V26+W26+X26+Y26+Z26)))</f>
+        <v/>
+      </c>
+      <c r="AX26" s="44" t="inlineStr">
+        <is>
+          <t>MODELED premium foiling fare</t>
+        </is>
+      </c>
+      <c r="AY26" s="44" t="inlineStr">
+        <is>
+          <t>MODELED tier demand</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="29" t="inlineStr">
+        <is>
+          <t>Eastern_Seaboard</t>
+        </is>
+      </c>
+      <c r="B27" s="29" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C27" s="30" t="inlineStr">
+        <is>
+          <t>Bangkok (Chao Phraya / Gulf gateway) → Pattaya (Bali Hai Pier)</t>
+        </is>
+      </c>
+      <c r="D27" s="31" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="E27" s="26" t="n">
+        <v>52</v>
+      </c>
+      <c r="F27" s="32" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
+      <c r="G27" s="32" t="inlineStr">
+        <is>
+          <t>low-med</t>
+        </is>
+      </c>
+      <c r="H27" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" s="33">
+        <f>60*D27/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J27" s="33">
+        <f>I27+turn_min+dwell_min</f>
+        <v/>
+      </c>
+      <c r="K27" s="34">
+        <f>MIN(15,FLOOR(60*service_hr/J27,1))</f>
+        <v/>
+      </c>
+      <c r="L27" s="34">
+        <f>ROUND(365*mech_uptime*H27,0)</f>
+        <v/>
+      </c>
+      <c r="M27" s="35">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="N27" s="35">
+        <f>revleg_sel</f>
+        <v/>
+      </c>
+      <c r="O27" s="34">
+        <f>ROUND(K27*L27*revleg_sel,0)</f>
+        <v/>
+      </c>
+      <c r="P27" s="36">
+        <f>load_sel</f>
+        <v/>
+      </c>
+      <c r="Q27" s="36">
+        <f>pax_cap*P27</f>
+        <v/>
+      </c>
+      <c r="R27" s="34">
+        <f>Q27*O27</f>
+        <v/>
+      </c>
+      <c r="S27" s="37">
+        <f>E27*discount</f>
+        <v/>
+      </c>
+      <c r="T27" s="38">
+        <f>S27*R27</f>
+        <v/>
+      </c>
+      <c r="U27" s="38">
+        <f>(battery/range_nm)*D27*O27*VLOOKUP(B27,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="V27" s="38">
+        <f>VLOOKUP(B27,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="W27" s="38">
+        <f>VLOOKUP(B27,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="X27" s="38">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Y27" s="38">
+        <f>VLOOKUP(B27,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="Z27" s="38">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AA27" s="38">
+        <f>U27+V27+W27+X27+Y27+Z27</f>
+        <v/>
+      </c>
+      <c r="AB27" s="38">
+        <f>VLOOKUP(B27,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AC27" s="38">
+        <f>T27-AA27</f>
+        <v/>
+      </c>
+      <c r="AD27" s="35">
+        <f>IF(T27=0,"",AC27/T27)</f>
+        <v/>
+      </c>
+      <c r="AE27" s="36">
+        <f>IF(AC27&lt;=0,"",VLOOKUP(B27,country_opex,7,FALSE)/AC27)</f>
+        <v/>
+      </c>
+      <c r="AF27" s="33">
+        <f>((D27*O27/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D27*O27*VLOOKUP(B27,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AG27" s="31" t="n">
+        <v>148000</v>
+      </c>
+      <c r="AH27" s="32" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="AI27" s="32" t="inlineStr">
+        <is>
+          <t>low-med</t>
+        </is>
+      </c>
+      <c r="AJ27" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AK27" s="34">
+        <f>IF(AG27="","",AG27*AJ27)</f>
+        <v/>
+      </c>
+      <c r="AL27" s="34">
+        <f>IF(OR(AG27="",R27=0),"",MIN(IF(AT27="",9.9E+99,AT27),FLOOR(AK27/R27,1)))</f>
+        <v/>
+      </c>
+      <c r="AM27" s="38">
+        <f>IF(AL27="","",AL27*T27)</f>
+        <v/>
+      </c>
+      <c r="AN27" s="36">
+        <f>IF(OR(AG27="",R27=0),"",MIN(IF(AT27="",9.9E+99,AT27),AK27/R27))</f>
+        <v/>
+      </c>
+      <c r="AO27" s="38">
+        <f>IF(AN27="","",AN27*T27)</f>
+        <v/>
+      </c>
+      <c r="AP27" s="40" t="n"/>
+      <c r="AQ27" s="32" t="inlineStr">
+        <is>
+          <t>Grounded</t>
+        </is>
+      </c>
+      <c r="AR27" s="41" t="n"/>
+      <c r="AS27" s="41" t="n"/>
+      <c r="AT27" s="42" t="n"/>
+      <c r="AU27" s="43">
+        <f>IF(((S27*pax_cap*load_thin*ROUND(K27*L27*revleg_thin,0))-(((battery/range_nm)*D27*ROUND(K27*L27*revleg_thin,0)*VLOOKUP(B27,country_opex,3,FALSE))+V27+W27+X27+Y27+Z27))&lt;=0,"",VLOOKUP(B27,country_opex,7,FALSE)/((S27*pax_cap*load_thin*ROUND(K27*L27*revleg_thin,0))-(((battery/range_nm)*D27*ROUND(K27*L27*revleg_thin,0)*VLOOKUP(B27,country_opex,3,FALSE))+V27+W27+X27+Y27+Z27)))</f>
+        <v/>
+      </c>
+      <c r="AV27" s="43">
+        <f>IF(((S27*pax_cap*load_mid*ROUND(K27*L27*revleg_mid,0))-(((battery/range_nm)*D27*ROUND(K27*L27*revleg_mid,0)*VLOOKUP(B27,country_opex,3,FALSE))+V27+W27+X27+Y27+Z27))&lt;=0,"",VLOOKUP(B27,country_opex,7,FALSE)/((S27*pax_cap*load_mid*ROUND(K27*L27*revleg_mid,0))-(((battery/range_nm)*D27*ROUND(K27*L27*revleg_mid,0)*VLOOKUP(B27,country_opex,3,FALSE))+V27+W27+X27+Y27+Z27)))</f>
+        <v/>
+      </c>
+      <c r="AW27" s="43">
+        <f>IF(((S27*pax_cap*load_full*ROUND(K27*L27*revleg_full,0))-(((battery/range_nm)*D27*ROUND(K27*L27*revleg_full,0)*VLOOKUP(B27,country_opex,3,FALSE))+V27+W27+X27+Y27+Z27))&lt;=0,"",VLOOKUP(B27,country_opex,7,FALSE)/((S27*pax_cap*load_full*ROUND(K27*L27*revleg_full,0))-(((battery/range_nm)*D27*ROUND(K27*L27*revleg_full,0)*VLOOKUP(B27,country_opex,3,FALSE))+V27+W27+X27+Y27+Z27)))</f>
+        <v/>
+      </c>
+      <c r="AX27" s="44" t="inlineStr">
+        <is>
+          <t>Premium slice of Bangkok-Pattaya leisure+EEC road flow; modeled pending operator validation.</t>
+        </is>
+      </c>
+      <c r="AY27" s="44" t="inlineStr">
+        <is>
+          <t>Premium slice of Bangkok-Pattaya leisure+EEC road flow; modeled pending operator validation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="29" t="inlineStr">
+        <is>
+          <t>Phuket</t>
+        </is>
+      </c>
+      <c r="B28" s="29" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C28" s="30" t="inlineStr">
+        <is>
+          <t>Phuket → Similan / Surin Islands</t>
+        </is>
+      </c>
+      <c r="D28" s="31" t="n">
+        <v>55</v>
+      </c>
+      <c r="E28" s="26" t="n">
+        <v>80</v>
+      </c>
+      <c r="F28" s="32" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="G28" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="H28" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I28" s="33">
+        <f>60*D28/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J28" s="33">
+        <f>I28+turn_min+dwell_min</f>
+        <v/>
+      </c>
+      <c r="K28" s="34">
+        <f>MIN(15,FLOOR(60*service_hr/J28,1))</f>
+        <v/>
+      </c>
+      <c r="L28" s="34">
+        <f>ROUND(365*mech_uptime*H28,0)</f>
+        <v/>
+      </c>
+      <c r="M28" s="35">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="N28" s="35">
+        <f>revleg_sel</f>
+        <v/>
+      </c>
+      <c r="O28" s="34">
+        <f>ROUND(K28*L28*revleg_sel,0)</f>
+        <v/>
+      </c>
+      <c r="P28" s="36">
+        <f>load_sel</f>
+        <v/>
+      </c>
+      <c r="Q28" s="36">
+        <f>pax_cap*P28</f>
+        <v/>
+      </c>
+      <c r="R28" s="34">
+        <f>Q28*O28</f>
+        <v/>
+      </c>
+      <c r="S28" s="37">
+        <f>E28*discount</f>
+        <v/>
+      </c>
+      <c r="T28" s="38">
+        <f>S28*R28</f>
+        <v/>
+      </c>
+      <c r="U28" s="38">
+        <f>(battery/range_nm)*D28*O28*VLOOKUP(B28,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="V28" s="38">
+        <f>VLOOKUP(B28,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="W28" s="38">
+        <f>VLOOKUP(B28,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="X28" s="38">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Y28" s="38">
+        <f>VLOOKUP(B28,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="Z28" s="38">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AA28" s="38">
+        <f>U28+V28+W28+X28+Y28+Z28</f>
+        <v/>
+      </c>
+      <c r="AB28" s="38">
+        <f>VLOOKUP(B28,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AC28" s="38">
+        <f>T28-AA28</f>
+        <v/>
+      </c>
+      <c r="AD28" s="35">
+        <f>IF(T28=0,"",AC28/T28)</f>
+        <v/>
+      </c>
+      <c r="AE28" s="36">
+        <f>IF(AC28&lt;=0,"",VLOOKUP(B28,country_opex,7,FALSE)/AC28)</f>
+        <v/>
+      </c>
+      <c r="AF28" s="33">
+        <f>((D28*O28/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D28*O28*VLOOKUP(B28,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AG28" s="31" t="n">
+        <v>580000</v>
+      </c>
+      <c r="AH28" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="AI28" s="32" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="AJ28" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AK28" s="34">
+        <f>IF(AG28="","",AG28*AJ28)</f>
+        <v/>
+      </c>
+      <c r="AL28" s="34">
+        <f>IF(OR(AG28="",R28=0),"",MIN(IF(AT28="",9.9E+99,AT28),FLOOR(AK28/R28,1)))</f>
+        <v/>
+      </c>
+      <c r="AM28" s="38">
+        <f>IF(AL28="","",AL28*T28)</f>
+        <v/>
+      </c>
+      <c r="AN28" s="36">
+        <f>IF(OR(AG28="",R28=0),"",MIN(IF(AT28="",9.9E+99,AT28),AK28/R28))</f>
+        <v/>
+      </c>
+      <c r="AO28" s="38">
+        <f>IF(AN28="","",AN28*T28)</f>
+        <v/>
+      </c>
+      <c r="AP28" s="40" t="n"/>
+      <c r="AQ28" s="32" t="inlineStr">
+        <is>
+          <t>Grounded</t>
+        </is>
+      </c>
+      <c r="AR28" s="41" t="n"/>
+      <c r="AS28" s="41" t="n"/>
+      <c r="AT28" s="42" t="n"/>
+      <c r="AU28" s="43">
+        <f>IF(((S28*pax_cap*load_thin*ROUND(K28*L28*revleg_thin,0))-(((battery/range_nm)*D28*ROUND(K28*L28*revleg_thin,0)*VLOOKUP(B28,country_opex,3,FALSE))+V28+W28+X28+Y28+Z28))&lt;=0,"",VLOOKUP(B28,country_opex,7,FALSE)/((S28*pax_cap*load_thin*ROUND(K28*L28*revleg_thin,0))-(((battery/range_nm)*D28*ROUND(K28*L28*revleg_thin,0)*VLOOKUP(B28,country_opex,3,FALSE))+V28+W28+X28+Y28+Z28)))</f>
+        <v/>
+      </c>
+      <c r="AV28" s="43">
+        <f>IF(((S28*pax_cap*load_mid*ROUND(K28*L28*revleg_mid,0))-(((battery/range_nm)*D28*ROUND(K28*L28*revleg_mid,0)*VLOOKUP(B28,country_opex,3,FALSE))+V28+W28+X28+Y28+Z28))&lt;=0,"",VLOOKUP(B28,country_opex,7,FALSE)/((S28*pax_cap*load_mid*ROUND(K28*L28*revleg_mid,0))-(((battery/range_nm)*D28*ROUND(K28*L28*revleg_mid,0)*VLOOKUP(B28,country_opex,3,FALSE))+V28+W28+X28+Y28+Z28)))</f>
+        <v/>
+      </c>
+      <c r="AW28" s="43">
+        <f>IF(((S28*pax_cap*load_full*ROUND(K28*L28*revleg_full,0))-(((battery/range_nm)*D28*ROUND(K28*L28*revleg_full,0)*VLOOKUP(B28,country_opex,3,FALSE))+V28+W28+X28+Y28+Z28))&lt;=0,"",VLOOKUP(B28,country_opex,7,FALSE)/((S28*pax_cap*load_full*ROUND(K28*L28*revleg_full,0))-(((battery/range_nm)*D28*ROUND(K28*L28*revleg_full,0)*VLOOKUP(B28,country_opex,3,FALSE))+V28+W28+X28+Y28+Z28)))</f>
+        <v/>
+      </c>
+      <c r="AX28" s="44" t="inlineStr">
+        <is>
           <t>Phuket-&gt;Similan/Surin premium shared speedboat day-tour (THB/USD 36): premium catamaran-speedboat tours ~2,500-2,600 THB incl 500 THB park fee+meals from Khao Lak (phiphitours 2,590 THB=$72); Phuket-origin runs higher ~2,900-3,500 THB ($80-97) for the longer 55nm leg. Private charter Phuket-&gt;Similan 50,000-80,000 THB/boat/day (forbesandpartners) = whole-boat, excluded. Premium per-seat anchored ~2,900 THB ($80) net for the longer Phuket origin.</t>
         </is>
       </c>
-      <c r="AY18" s="44" t="inlineStr">
+      <c r="AY28" s="44" t="inlineStr">
         <is>
           <t>Mu Ko Similan NP official visitor statistics (DNP/park clarification, May-2025, via MGR Online https://mgronline.com/uptodate/detail/9680000041761): FY2561(2018)=912,566; FY2562(2019)=676,793; FY2566(2023)=352,701; FY2567(2024)=578,535; FY2568=503,142 as of 30-Apr-2025. Daily cap 3,850 visitors/day (DNP, http://news.dnp.go.th/news/7966). Season: park CLOSED ~May 16 - Oct 14; open season ~212 days/yr (reopened 15-Oct each year, prd.go.th).</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="45" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="29" t="inlineStr">
+        <is>
+          <t>Royal_Coast</t>
+        </is>
+      </c>
+      <c r="B29" s="29" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C29" s="30" t="inlineStr">
+        <is>
+          <t>Hua Hin (pier) → Pattaya (Bali Hai Pier)</t>
+        </is>
+      </c>
+      <c r="D29" s="31" t="n">
+        <v>57.2</v>
+      </c>
+      <c r="E29" s="26" t="n">
+        <v>78</v>
+      </c>
+      <c r="F29" s="32" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
+      <c r="G29" s="32" t="inlineStr">
+        <is>
+          <t>low-med</t>
+        </is>
+      </c>
+      <c r="H29" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I29" s="33">
+        <f>60*D29/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J29" s="33">
+        <f>I29+turn_min+dwell_min</f>
+        <v/>
+      </c>
+      <c r="K29" s="34">
+        <f>MIN(15,FLOOR(60*service_hr/J29,1))</f>
+        <v/>
+      </c>
+      <c r="L29" s="34">
+        <f>ROUND(365*mech_uptime*H29,0)</f>
+        <v/>
+      </c>
+      <c r="M29" s="35">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="N29" s="35">
+        <f>revleg_sel</f>
+        <v/>
+      </c>
+      <c r="O29" s="34">
+        <f>ROUND(K29*L29*revleg_sel,0)</f>
+        <v/>
+      </c>
+      <c r="P29" s="36">
+        <f>load_sel</f>
+        <v/>
+      </c>
+      <c r="Q29" s="36">
+        <f>pax_cap*P29</f>
+        <v/>
+      </c>
+      <c r="R29" s="34">
+        <f>Q29*O29</f>
+        <v/>
+      </c>
+      <c r="S29" s="37">
+        <f>E29*discount</f>
+        <v/>
+      </c>
+      <c r="T29" s="38">
+        <f>S29*R29</f>
+        <v/>
+      </c>
+      <c r="U29" s="38">
+        <f>(battery/range_nm)*D29*O29*VLOOKUP(B29,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="V29" s="38">
+        <f>VLOOKUP(B29,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="W29" s="38">
+        <f>VLOOKUP(B29,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="X29" s="38">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Y29" s="38">
+        <f>VLOOKUP(B29,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="Z29" s="38">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AA29" s="38">
+        <f>U29+V29+W29+X29+Y29+Z29</f>
+        <v/>
+      </c>
+      <c r="AB29" s="38">
+        <f>VLOOKUP(B29,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AC29" s="38">
+        <f>T29-AA29</f>
+        <v/>
+      </c>
+      <c r="AD29" s="35">
+        <f>IF(T29=0,"",AC29/T29)</f>
+        <v/>
+      </c>
+      <c r="AE29" s="36">
+        <f>IF(AC29&lt;=0,"",VLOOKUP(B29,country_opex,7,FALSE)/AC29)</f>
+        <v/>
+      </c>
+      <c r="AF29" s="33">
+        <f>((D29*O29/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D29*O29*VLOOKUP(B29,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AG29" s="31" t="n">
+        <v>52000</v>
+      </c>
+      <c r="AH29" s="32" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="AI29" s="32" t="inlineStr">
+        <is>
+          <t>low-med</t>
+        </is>
+      </c>
+      <c r="AJ29" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AK29" s="34">
+        <f>IF(AG29="","",AG29*AJ29)</f>
+        <v/>
+      </c>
+      <c r="AL29" s="34">
+        <f>IF(OR(AG29="",R29=0),"",MIN(IF(AT29="",9.9E+99,AT29),FLOOR(AK29/R29,1)))</f>
+        <v/>
+      </c>
+      <c r="AM29" s="38">
+        <f>IF(AL29="","",AL29*T29)</f>
+        <v/>
+      </c>
+      <c r="AN29" s="36">
+        <f>IF(OR(AG29="",R29=0),"",MIN(IF(AT29="",9.9E+99,AT29),AK29/R29))</f>
+        <v/>
+      </c>
+      <c r="AO29" s="38">
+        <f>IF(AN29="","",AN29*T29)</f>
+        <v/>
+      </c>
+      <c r="AP29" s="40" t="n"/>
+      <c r="AQ29" s="32" t="inlineStr">
+        <is>
+          <t>Grounded</t>
+        </is>
+      </c>
+      <c r="AR29" s="41" t="n"/>
+      <c r="AS29" s="41" t="n"/>
+      <c r="AT29" s="42" t="n"/>
+      <c r="AU29" s="43">
+        <f>IF(((S29*pax_cap*load_thin*ROUND(K29*L29*revleg_thin,0))-(((battery/range_nm)*D29*ROUND(K29*L29*revleg_thin,0)*VLOOKUP(B29,country_opex,3,FALSE))+V29+W29+X29+Y29+Z29))&lt;=0,"",VLOOKUP(B29,country_opex,7,FALSE)/((S29*pax_cap*load_thin*ROUND(K29*L29*revleg_thin,0))-(((battery/range_nm)*D29*ROUND(K29*L29*revleg_thin,0)*VLOOKUP(B29,country_opex,3,FALSE))+V29+W29+X29+Y29+Z29)))</f>
+        <v/>
+      </c>
+      <c r="AV29" s="43">
+        <f>IF(((S29*pax_cap*load_mid*ROUND(K29*L29*revleg_mid,0))-(((battery/range_nm)*D29*ROUND(K29*L29*revleg_mid,0)*VLOOKUP(B29,country_opex,3,FALSE))+V29+W29+X29+Y29+Z29))&lt;=0,"",VLOOKUP(B29,country_opex,7,FALSE)/((S29*pax_cap*load_mid*ROUND(K29*L29*revleg_mid,0))-(((battery/range_nm)*D29*ROUND(K29*L29*revleg_mid,0)*VLOOKUP(B29,country_opex,3,FALSE))+V29+W29+X29+Y29+Z29)))</f>
+        <v/>
+      </c>
+      <c r="AW29" s="43">
+        <f>IF(((S29*pax_cap*load_full*ROUND(K29*L29*revleg_full,0))-(((battery/range_nm)*D29*ROUND(K29*L29*revleg_full,0)*VLOOKUP(B29,country_opex,3,FALSE))+V29+W29+X29+Y29+Z29))&lt;=0,"",VLOOKUP(B29,country_opex,7,FALSE)/((S29*pax_cap*load_full*ROUND(K29*L29*revleg_full,0))-(((battery/range_nm)*D29*ROUND(K29*L29*revleg_full,0)*VLOOKUP(B29,country_opex,3,FALSE))+V29+W29+X29+Y29+Z29)))</f>
+        <v/>
+      </c>
+      <c r="AX29" s="44" t="inlineStr">
+        <is>
+          <t>East-West Ferry Project validated cross-Gulf demand; foiling premium tier.</t>
+        </is>
+      </c>
+      <c r="AY29" s="44" t="inlineStr">
+        <is>
+          <t>East-West Ferry Project validated cross-Gulf demand; foiling premium tier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="45" t="inlineStr">
         <is>
           <t>TOTAL / median</t>
         </is>
       </c>
-      <c r="T19" s="46">
-        <f>SUM(T4:T18)</f>
-        <v/>
-      </c>
-      <c r="AC19" s="46">
-        <f>SUM(AC4:AC18)</f>
-        <v/>
-      </c>
-      <c r="AD19" s="47">
-        <f>IF(T19=0,"",AC19/T19)</f>
-        <v/>
-      </c>
-      <c r="AL19" s="48">
-        <f>SUM(AL4:AL18)</f>
-        <v/>
-      </c>
-      <c r="AM19" s="46">
-        <f>SUM(AM4:AM18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="T30" s="46">
+        <f>SUM(T4:T29)</f>
+        <v/>
+      </c>
+      <c r="AC30" s="46">
+        <f>SUM(AC4:AC29)</f>
+        <v/>
+      </c>
+      <c r="AD30" s="47">
+        <f>IF(T30=0,"",AC30/T30)</f>
+        <v/>
+      </c>
+      <c r="AL30" s="48">
+        <f>SUM(AL4:AL29)</f>
+        <v/>
+      </c>
+      <c r="AM30" s="46">
+        <f>SUM(AM4:AM29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>Market fleet build-up — grounded floor (network-sum of raw vessel fractions per market, rounded once; subset slices excluded; legacy per-corridor-floor totals above kept for reference)</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="24" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="24" t="inlineStr">
         <is>
           <t>Market</t>
         </is>
       </c>
-      <c r="B22" s="24" t="inlineStr">
+      <c r="B33" s="24" t="inlineStr">
         <is>
           <t>Fleet basis</t>
         </is>
       </c>
-      <c r="C22" s="24" t="inlineStr">
+      <c r="C33" s="24" t="inlineStr">
         <is>
           <t>Raw vessels (sum)</t>
         </is>
       </c>
-      <c r="D22" s="24" t="inlineStr">
+      <c r="D33" s="24" t="inlineStr">
         <is>
           <t>Fleet (rounded once)</t>
         </is>
       </c>
-      <c r="E22" s="24" t="inlineStr">
+      <c r="E33" s="24" t="inlineStr">
         <is>
           <t>Market rev/yr (raw sum)</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="25" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="25" t="inlineStr">
         <is>
           <t>Bangkok</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B34" s="13" t="inlineStr">
         <is>
           <t>network_sum / ceil</t>
         </is>
       </c>
-      <c r="C23" s="23">
-        <f>SUMIFS(AN4:AN18,A4:A18,"Bangkok",AP4:AP18,"=",AQ4:AQ18,"Grounded")</f>
-        <v/>
-      </c>
-      <c r="D23" s="49">
-        <f>IF(C23=0,0,CEILING(C23,1))</f>
-        <v/>
-      </c>
-      <c r="E23" s="50">
-        <f>SUMIFS(AO4:AO18,A4:A18,"Bangkok",AP4:AP18,"=",AQ4:AQ18,"Grounded")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="25" t="inlineStr">
+      <c r="C34" s="23">
+        <f>SUMIFS(AN4:AN29,A4:A29,"Bangkok",AP4:AP29,"=",AQ4:AQ29,"Grounded")</f>
+        <v/>
+      </c>
+      <c r="D34" s="49">
+        <f>IF(C34=0,0,CEILING(C34,1))</f>
+        <v/>
+      </c>
+      <c r="E34" s="50">
+        <f>SUMIFS(AO4:AO29,A4:A29,"Bangkok",AP4:AP29,"=",AQ4:AQ29,"Grounded")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="25" t="inlineStr">
+        <is>
+          <t>Eastern_Seaboard</t>
+        </is>
+      </c>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>network_sum / ceil</t>
+        </is>
+      </c>
+      <c r="C35" s="23">
+        <f>SUMIFS(AN4:AN29,A4:A29,"Eastern_Seaboard",AP4:AP29,"=",AQ4:AQ29,"Grounded")</f>
+        <v/>
+      </c>
+      <c r="D35" s="49">
+        <f>IF(C35=0,0,CEILING(C35,1))</f>
+        <v/>
+      </c>
+      <c r="E35" s="50">
+        <f>SUMIFS(AO4:AO29,A4:A29,"Eastern_Seaboard",AP4:AP29,"=",AQ4:AQ29,"Grounded")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="25" t="inlineStr">
         <is>
           <t>Koh Samui</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B36" s="13" t="inlineStr">
         <is>
           <t>network_sum / ceil</t>
         </is>
       </c>
-      <c r="C24" s="23">
-        <f>SUMIFS(AN4:AN18,A4:A18,"Koh Samui",AP4:AP18,"=",AQ4:AQ18,"Grounded")</f>
-        <v/>
-      </c>
-      <c r="D24" s="49">
-        <f>IF(C24=0,0,CEILING(C24,1))</f>
-        <v/>
-      </c>
-      <c r="E24" s="50">
-        <f>SUMIFS(AO4:AO18,A4:A18,"Koh Samui",AP4:AP18,"=",AQ4:AQ18,"Grounded")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="25" t="inlineStr">
+      <c r="C36" s="23">
+        <f>SUMIFS(AN4:AN29,A4:A29,"Koh Samui",AP4:AP29,"=",AQ4:AQ29,"Grounded")</f>
+        <v/>
+      </c>
+      <c r="D36" s="49">
+        <f>IF(C36=0,0,CEILING(C36,1))</f>
+        <v/>
+      </c>
+      <c r="E36" s="50">
+        <f>SUMIFS(AO4:AO29,A4:A29,"Koh Samui",AP4:AP29,"=",AQ4:AQ29,"Grounded")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="25" t="inlineStr">
         <is>
           <t>Phuket</t>
         </is>
       </c>
-      <c r="B25" s="13" t="inlineStr">
+      <c r="B37" s="13" t="inlineStr">
         <is>
           <t>network_sum / ceil</t>
         </is>
       </c>
-      <c r="C25" s="23">
-        <f>SUMIFS(AN4:AN18,A4:A18,"Phuket",AP4:AP18,"=",AQ4:AQ18,"Grounded")</f>
-        <v/>
-      </c>
-      <c r="D25" s="49">
-        <f>IF(C25=0,0,CEILING(C25,1))</f>
-        <v/>
-      </c>
-      <c r="E25" s="50">
-        <f>SUMIFS(AO4:AO18,A4:A18,"Phuket",AP4:AP18,"=",AQ4:AQ18,"Grounded")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="45" t="inlineStr">
+      <c r="C37" s="23">
+        <f>SUMIFS(AN4:AN29,A4:A29,"Phuket",AP4:AP29,"=",AQ4:AQ29,"Grounded")</f>
+        <v/>
+      </c>
+      <c r="D37" s="49">
+        <f>IF(C37=0,0,CEILING(C37,1))</f>
+        <v/>
+      </c>
+      <c r="E37" s="50">
+        <f>SUMIFS(AO4:AO29,A4:A29,"Phuket",AP4:AP29,"=",AQ4:AQ29,"Grounded")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="25" t="inlineStr">
+        <is>
+          <t>Royal_Coast</t>
+        </is>
+      </c>
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>network_sum / ceil</t>
+        </is>
+      </c>
+      <c r="C38" s="23">
+        <f>SUMIFS(AN4:AN29,A4:A29,"Royal_Coast",AP4:AP29,"=",AQ4:AQ29,"Grounded")</f>
+        <v/>
+      </c>
+      <c r="D38" s="49">
+        <f>IF(C38=0,0,CEILING(C38,1))</f>
+        <v/>
+      </c>
+      <c r="E38" s="50">
+        <f>SUMIFS(AO4:AO29,A4:A29,"Royal_Coast",AP4:AP29,"=",AQ4:AQ29,"Grounded")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="45" t="inlineStr">
         <is>
           <t>GROUNDED FLOOR (PUBLISHED)</t>
         </is>
       </c>
-      <c r="D26" s="48">
-        <f>SUM(D23:D25)</f>
-        <v/>
-      </c>
-      <c r="E26" s="46">
-        <f>SUM(E23:E25)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="20" t="inlineStr">
+      <c r="D39" s="48">
+        <f>SUM(D34:D38)</f>
+        <v/>
+      </c>
+      <c r="E39" s="46">
+        <f>SUM(E34:E38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="20" t="inlineStr">
         <is>
           <t>ESTIMATED DEMAND (country-median cascade; held OUT of grounded floor)</t>
         </is>
       </c>
-      <c r="D27" s="51">
-        <f>SUMIF(AQ4:AQ18,"Estimated",AL4:AL18)</f>
-        <v/>
-      </c>
-      <c r="E27" s="52">
-        <f>SUMIF(AQ4:AQ18,"Estimated",AM4:AM18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="53" t="inlineStr">
+      <c r="D40" s="51">
+        <f>SUMIF(AQ4:AQ29,"Estimated",AL4:AL29)</f>
+        <v/>
+      </c>
+      <c r="E40" s="52">
+        <f>SUMIF(AQ4:AQ29,"Estimated",AM4:AM29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="53" t="inlineStr">
         <is>
           <t>Held for Quanta-LR (&gt;70nm, roadmap H2 2026+):</t>
         </is>
       </c>
-      <c r="C28" s="54" t="inlineStr">
+      <c r="C41" s="54" t="inlineStr">
         <is>
           <t>Phuket → Langkawi (cross-border, regional reach) (107nm)</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="C29" s="54" t="inlineStr">
+    <row r="42">
+      <c r="C42" s="54" t="inlineStr">
         <is>
           <t>Phuket → Langkawi (cross-border, regional reach) (107nm)</t>
         </is>
@@ -5310,8 +7547,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A21:L21"/>
     <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A32:L32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5480,11 +7717,11 @@
         </is>
       </c>
       <c r="C11" s="39" t="n">
-        <v>0.0968</v>
+        <v>0.1056</v>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>New-entrant ~10% share of today's pool (= the published floor).</t>
+          <t>New-entrant ~11% share of today's pool (= the published floor).</t>
         </is>
       </c>
     </row>
@@ -5557,7 +7794,7 @@
     <row r="18">
       <c r="A18" s="25" t="inlineStr">
         <is>
-          <t>SOM full network (~10% capture, today, +greenfield)</t>
+          <t>SOM full network (~11% capture, today, +greenfield)</t>
         </is>
       </c>
       <c r="B18" s="50">
@@ -5574,7 +7811,7 @@
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>Floor posture (~10% captive capture, today's demand) extended across the whole mapped network.</t>
+          <t>Floor posture (~11% captive capture, today's demand) extended across the whole mapped network.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(grab-thailand): cascade economics for BKK↔Hua Hin marquee corridor
Adds rn-01f164a3d43c to depth demand (85k pax, $68 fare). At 88nm the leg
is framed Quanta-LR roadmap per 70nm Pioneer gate; geometry remains sealed.
</commit_message>
<xml_diff>
--- a/finance/_refresh_grab-thailand.xlsx
+++ b/finance/_refresh_grab-thailand.xlsx
@@ -1919,7 +1919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY42"/>
+  <dimension ref="A1:AY43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7545,6 +7545,13 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="C43" s="54" t="inlineStr">
+        <is>
+          <t>Bangkok (ICONSIAM / Chao Phraya) → Hua Hin (pier) (88.0nm)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:L1"/>

</xml_diff>